<commit_message>
automate zo docs and add crystallizer
</commit_message>
<xml_diff>
--- a/docs/technical_reference/unit_models/zero_order_unit_models/WT3_unit_classification_for_doc.xlsx
+++ b/docs/technical_reference/unit_models/zero_order_unit_models/WT3_unit_classification_for_doc.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10517"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F54105F9-699E-40C1-91E9-7B98EAFB177C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35874F6C-7701-DF4B-AA7A-C888519018C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,7 @@
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$93</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="999" uniqueCount="512">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="515">
   <si>
     <t>Name</t>
   </si>
@@ -1568,6 +1568,15 @@
   </si>
   <si>
     <t>cost_electrocoagulation</t>
+  </si>
+  <si>
+    <t>crystallizer_zo</t>
+  </si>
+  <si>
+    <t>CrystallizerZO</t>
+  </si>
+  <si>
+    <t>cost_crystallizer</t>
   </si>
 </sst>
 </file>
@@ -1655,9 +1664,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1695,9 +1704,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1730,26 +1739,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1782,26 +1774,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1975,21 +1950,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J92"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:J93"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="33.46484375" customWidth="1"/>
+    <col min="1" max="1" width="33.5" customWidth="1"/>
     <col min="2" max="2" width="37.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="10.53125" customWidth="1"/>
+    <col min="4" max="4" width="10.5" customWidth="1"/>
     <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.19921875" customWidth="1"/>
-    <col min="8" max="8" width="38.53125" customWidth="1"/>
-    <col min="9" max="9" width="30.19921875" customWidth="1"/>
-    <col min="10" max="10" width="25.53125" customWidth="1"/>
+    <col min="7" max="7" width="20.1640625" customWidth="1"/>
+    <col min="8" max="8" width="38.5" customWidth="1"/>
+    <col min="9" max="9" width="30.1640625" customWidth="1"/>
+    <col min="10" max="10" width="25.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2021,7 +1996,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -2048,15 +2023,15 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I2" t="str">
-        <f t="shared" ref="I2:I38" si="1">IF(E2="SIDO","single-input, double-output",IF(E2="SISO","single-input, single-output",IF(E2="PT","pass-through",IF(E2="DISO","double-input, single-output",IF(E2="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
+        <f t="shared" ref="I2:I39" si="1">IF(E2="SIDO","single-input, double-output",IF(E2="SISO","single-input, single-output",IF(E2="PT","pass-through",IF(E2="DISO","double-input, single-output",IF(E2="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
         <v>single-input, double-output</v>
       </c>
       <c r="J2" t="str">
-        <f t="shared" ref="J2:J38" si="2">IF(E2="SIDO","sido_methods",IF(E2="SISO","siso_methods",IF(E2="PT","pt_methods",IF(E2="DISO","diso_methods",IF(E2="SIDO reactive","sidor_methods","")))))</f>
+        <f t="shared" ref="J2:J39" si="2">IF(E2="SIDO","sido_methods",IF(E2="SISO","siso_methods",IF(E2="PT","pt_methods",IF(E2="DISO","diso_methods",IF(E2="SIDO reactive","sidor_methods","")))))</f>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -2091,7 +2066,7 @@
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>506</v>
       </c>
@@ -2126,7 +2101,7 @@
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>463</v>
       </c>
@@ -2160,7 +2135,7 @@
         <v>sidor_methods</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -2194,7 +2169,7 @@
         <v>sidor_methods</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>465</v>
       </c>
@@ -2228,7 +2203,7 @@
         <v>sidor_methods</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -2263,7 +2238,7 @@
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -2298,7 +2273,7 @@
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -2333,7 +2308,7 @@
         <v>siso_methods</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>372</v>
       </c>
@@ -2368,7 +2343,7 @@
         <v>pt_methods</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -2402,7 +2377,7 @@
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>33</v>
       </c>
@@ -2437,7 +2412,7 @@
         <v>pt_methods</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>35</v>
       </c>
@@ -2471,7 +2446,7 @@
         <v>sidor_methods</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>38</v>
       </c>
@@ -2506,7 +2481,7 @@
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>467</v>
       </c>
@@ -2540,7 +2515,7 @@
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>40</v>
       </c>
@@ -2574,7 +2549,7 @@
         <v>pt_methods</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>43</v>
       </c>
@@ -2608,7 +2583,7 @@
         <v>siso_methods</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>46</v>
       </c>
@@ -2643,7 +2618,7 @@
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>471</v>
       </c>
@@ -2677,7 +2652,7 @@
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>48</v>
       </c>
@@ -2712,7 +2687,7 @@
         <v>pt_methods</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>50</v>
       </c>
@@ -2746,7 +2721,7 @@
         <v>pt_methods</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>53</v>
       </c>
@@ -2780,7 +2755,7 @@
         <v>sidor_methods</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>55</v>
       </c>
@@ -2814,7 +2789,7 @@
         <v>siso_methods</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>59</v>
       </c>
@@ -2849,7 +2824,7 @@
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>61</v>
       </c>
@@ -2884,7 +2859,7 @@
         <v>pt_methods</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>63</v>
       </c>
@@ -2918,256 +2893,256 @@
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" t="s">
+        <v>512</v>
+      </c>
+      <c r="C28" t="s">
+        <v>513</v>
+      </c>
+      <c r="D28" t="s">
+        <v>30</v>
+      </c>
+      <c r="E28" t="s">
+        <v>11</v>
+      </c>
+      <c r="F28" t="b">
+        <v>0</v>
+      </c>
+      <c r="G28" t="s">
+        <v>31</v>
+      </c>
+      <c r="H28" t="s">
+        <v>514</v>
+      </c>
+      <c r="I28" t="str">
+        <f t="shared" ref="I28" si="3">IF(E28="SIDO","single-input, double-output",IF(E28="SISO","single-input, single-output",IF(E28="PT","pass-through",IF(E28="DISO","double-input, single-output",IF(E28="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
+        <v>single-input, double-output</v>
+      </c>
+      <c r="J28" t="str">
+        <f t="shared" ref="J28" si="4">IF(E28="SIDO","sido_methods",IF(E28="SISO","siso_methods",IF(E28="PT","pt_methods",IF(E28="DISO","diso_methods",IF(E28="SIDO reactive","sidor_methods","")))))</f>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
         <v>66</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B29" t="s">
         <v>67</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C29" t="s">
         <v>391</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D29" t="s">
         <v>10</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E29" t="s">
         <v>26</v>
       </c>
-      <c r="F28" t="b">
+      <c r="F29" t="b">
         <v>1</v>
       </c>
-      <c r="G28" t="s">
+      <c r="G29" t="s">
         <v>12</v>
       </c>
-      <c r="H28" t="str">
-        <f>IF(D28="basic","cost_power_law_flow")</f>
+      <c r="H29" t="str">
+        <f>IF(D29="basic","cost_power_law_flow")</f>
         <v>cost_power_law_flow</v>
       </c>
-      <c r="I28" t="str">
+      <c r="I29" t="str">
         <f t="shared" si="1"/>
         <v>single-input, single-output</v>
       </c>
-      <c r="J28" t="str">
+      <c r="J29" t="str">
         <f t="shared" si="2"/>
         <v>siso_methods</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A29" t="s">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
         <v>68</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B30" t="s">
         <v>69</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C30" t="s">
         <v>380</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D30" t="s">
         <v>30</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E30" t="s">
         <v>27</v>
       </c>
-      <c r="F29" t="b">
+      <c r="F30" t="b">
         <v>1</v>
       </c>
-      <c r="G29" t="s">
+      <c r="G30" t="s">
         <v>21</v>
       </c>
-      <c r="H29" t="s">
+      <c r="H30" t="s">
         <v>70</v>
       </c>
-      <c r="I29" t="str">
+      <c r="I30" t="str">
         <f t="shared" si="1"/>
         <v>pass-through</v>
       </c>
-      <c r="J29" t="str">
+      <c r="J30" t="str">
         <f t="shared" si="2"/>
         <v>pt_methods</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A30" t="s">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
         <v>71</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B31" t="s">
         <v>72</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C31" t="s">
         <v>392</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D31" t="s">
         <v>10</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E31" t="s">
         <v>11</v>
       </c>
-      <c r="F30" t="b">
+      <c r="F31" t="b">
         <v>1</v>
       </c>
-      <c r="G30" t="s">
+      <c r="G31" t="s">
         <v>12</v>
       </c>
-      <c r="H30" t="str">
-        <f>IF(D30="basic","cost_power_law_flow")</f>
+      <c r="H31" t="str">
+        <f>IF(D31="basic","cost_power_law_flow")</f>
         <v>cost_power_law_flow</v>
       </c>
-      <c r="I30" t="str">
+      <c r="I31" t="str">
         <f t="shared" si="1"/>
         <v>single-input, double-output</v>
       </c>
-      <c r="J30" t="str">
+      <c r="J31" t="str">
         <f t="shared" si="2"/>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A31" t="s">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
         <v>73</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B32" t="s">
         <v>74</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C32" t="s">
         <v>381</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D32" t="s">
         <v>57</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E32" t="s">
         <v>18</v>
       </c>
-      <c r="F31" t="b">
+      <c r="F32" t="b">
         <v>1</v>
       </c>
-      <c r="G31" t="s">
+      <c r="G32" t="s">
         <v>12</v>
       </c>
-      <c r="H31" t="s">
+      <c r="H32" t="s">
         <v>75</v>
       </c>
-      <c r="I31" t="str">
+      <c r="I32" t="str">
         <f t="shared" si="1"/>
         <v>reactive single-inlet, double-outlet</v>
       </c>
-      <c r="J31" t="str">
+      <c r="J32" t="str">
         <f t="shared" si="2"/>
         <v>sidor_methods</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A32" t="s">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
         <v>76</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B33" t="s">
         <v>77</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C33" t="s">
         <v>430</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D33" t="s">
         <v>10</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E33" t="s">
         <v>11</v>
       </c>
-      <c r="F32" t="b">
+      <c r="F33" t="b">
         <v>1</v>
       </c>
-      <c r="G32" t="s">
+      <c r="G33" t="s">
         <v>12</v>
       </c>
-      <c r="H32" t="str">
-        <f>IF(D32="basic","cost_power_law_flow")</f>
+      <c r="H33" t="str">
+        <f>IF(D33="basic","cost_power_law_flow")</f>
         <v>cost_power_law_flow</v>
       </c>
-      <c r="I32" t="str">
+      <c r="I33" t="str">
         <f t="shared" si="1"/>
         <v>single-input, double-output</v>
       </c>
-      <c r="J32" t="str">
+      <c r="J33" t="str">
         <f t="shared" si="2"/>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A33" t="s">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
         <v>78</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B34" t="s">
         <v>79</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C34" t="s">
         <v>395</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D34" t="s">
         <v>30</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E34" t="s">
         <v>18</v>
       </c>
-      <c r="F33" t="b">
+      <c r="F34" t="b">
         <v>0</v>
       </c>
-      <c r="G33" t="s">
+      <c r="G34" t="s">
         <v>31</v>
       </c>
-      <c r="H33" t="s">
+      <c r="H34" t="s">
         <v>80</v>
       </c>
-      <c r="I33" t="str">
+      <c r="I34" t="str">
         <f t="shared" si="1"/>
         <v>reactive single-inlet, double-outlet</v>
       </c>
-      <c r="J33" t="str">
+      <c r="J34" t="str">
         <f t="shared" si="2"/>
         <v>sidor_methods</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A34" t="s">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
         <v>508</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B35" t="s">
         <v>509</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C35" t="s">
         <v>510</v>
-      </c>
-      <c r="D34" t="s">
-        <v>30</v>
-      </c>
-      <c r="E34" t="s">
-        <v>11</v>
-      </c>
-      <c r="F34" t="b">
-        <v>0</v>
-      </c>
-      <c r="G34" t="s">
-        <v>31</v>
-      </c>
-      <c r="H34" t="s">
-        <v>511</v>
-      </c>
-      <c r="I34" t="str">
-        <f t="shared" si="1"/>
-        <v>single-input, double-output</v>
-      </c>
-      <c r="J34" t="str">
-        <f t="shared" si="2"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A35" t="s">
-        <v>81</v>
-      </c>
-      <c r="B35" t="s">
-        <v>82</v>
-      </c>
-      <c r="C35" t="s">
-        <v>382</v>
       </c>
       <c r="D35" t="s">
         <v>30</v>
@@ -3182,7 +3157,7 @@
         <v>31</v>
       </c>
       <c r="H35" t="s">
-        <v>65</v>
+        <v>511</v>
       </c>
       <c r="I35" t="str">
         <f t="shared" si="1"/>
@@ -3193,56 +3168,55 @@
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B36" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C36" t="s">
-        <v>396</v>
+        <v>382</v>
       </c>
       <c r="D36" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E36" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G36" t="s">
-        <v>12</v>
-      </c>
-      <c r="H36" t="str">
-        <f>IF(D36="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+        <v>31</v>
+      </c>
+      <c r="H36" t="s">
+        <v>65</v>
       </c>
       <c r="I36" t="str">
         <f t="shared" si="1"/>
-        <v>pass-through</v>
+        <v>single-input, double-output</v>
       </c>
       <c r="J36" t="str">
         <f t="shared" si="2"/>
-        <v>pt_methods</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.45">
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B37" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C37" t="s">
-        <v>437</v>
+        <v>396</v>
       </c>
       <c r="D37" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E37" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F37" t="b">
         <v>1</v>
@@ -3250,33 +3224,34 @@
       <c r="G37" t="s">
         <v>12</v>
       </c>
-      <c r="H37" t="s">
-        <v>87</v>
+      <c r="H37" t="str">
+        <f>IF(D37="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I37" t="str">
         <f t="shared" si="1"/>
-        <v>single-input, double-output</v>
+        <v>pass-through</v>
       </c>
       <c r="J37" t="str">
         <f t="shared" si="2"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.45">
+        <v>pt_methods</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B38" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C38" t="s">
-        <v>393</v>
+        <v>437</v>
       </c>
       <c r="D38" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E38" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F38" t="b">
         <v>1</v>
@@ -3284,163 +3259,163 @@
       <c r="G38" t="s">
         <v>12</v>
       </c>
-      <c r="H38" t="str">
-        <f>IF(D38="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H38" t="s">
+        <v>87</v>
       </c>
       <c r="I38" t="str">
         <f t="shared" si="1"/>
-        <v>pass-through</v>
+        <v>single-input, double-output</v>
       </c>
       <c r="J38" t="str">
         <f t="shared" si="2"/>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>88</v>
+      </c>
+      <c r="B39" t="s">
+        <v>89</v>
+      </c>
+      <c r="C39" t="s">
+        <v>393</v>
+      </c>
+      <c r="D39" t="s">
+        <v>10</v>
+      </c>
+      <c r="E39" t="s">
+        <v>27</v>
+      </c>
+      <c r="F39" t="b">
+        <v>1</v>
+      </c>
+      <c r="G39" t="s">
+        <v>12</v>
+      </c>
+      <c r="H39" t="str">
+        <f>IF(D39="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
+      </c>
+      <c r="I39" t="str">
+        <f t="shared" si="1"/>
+        <v>pass-through</v>
+      </c>
+      <c r="J39" t="str">
+        <f t="shared" si="2"/>
         <v>pt_methods</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A39" t="s">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
         <v>90</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B40" t="s">
         <v>91</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C40" t="s">
         <v>394</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D40" t="s">
         <v>92</v>
       </c>
-      <c r="E39" t="s">
+      <c r="E40" t="s">
         <v>58</v>
-      </c>
-      <c r="F39" t="b">
-        <v>0</v>
-      </c>
-      <c r="G39" t="s">
-        <v>58</v>
-      </c>
-      <c r="H39" t="b">
-        <f>IF(D39="basic","cost_power_law_flow")</f>
-        <v>0</v>
-      </c>
-      <c r="I39" t="s">
-        <v>93</v>
-      </c>
-      <c r="J39" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A40" t="s">
-        <v>94</v>
-      </c>
-      <c r="B40" t="s">
-        <v>95</v>
-      </c>
-      <c r="C40" t="s">
-        <v>438</v>
-      </c>
-      <c r="D40" t="s">
-        <v>30</v>
-      </c>
-      <c r="E40" t="s">
-        <v>11</v>
       </c>
       <c r="F40" t="b">
         <v>0</v>
       </c>
       <c r="G40" t="s">
-        <v>31</v>
-      </c>
-      <c r="H40" t="s">
-        <v>96</v>
-      </c>
-      <c r="I40" t="str">
-        <f t="shared" ref="I40:I45" si="3">IF(E40="SIDO","single-input, double-output",IF(E40="SISO","single-input, single-output",IF(E40="PT","pass-through",IF(E40="DISO","double-input, single-output",IF(E40="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
-        <v>single-input, double-output</v>
-      </c>
-      <c r="J40" t="str">
-        <f t="shared" ref="J40:J45" si="4">IF(E40="SIDO","sido_methods",IF(E40="SISO","siso_methods",IF(E40="PT","pt_methods",IF(E40="DISO","diso_methods",IF(E40="SIDO reactive","sidor_methods","")))))</f>
-        <v>sido_methods</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.45">
+        <v>58</v>
+      </c>
+      <c r="H40" t="b">
+        <f>IF(D40="basic","cost_power_law_flow")</f>
+        <v>0</v>
+      </c>
+      <c r="I40" t="s">
+        <v>93</v>
+      </c>
+      <c r="J40" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B41" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C41" t="s">
-        <v>423</v>
+        <v>438</v>
       </c>
       <c r="D41" t="s">
         <v>30</v>
       </c>
       <c r="E41" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G41" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="H41" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="I41" t="str">
-        <f t="shared" si="3"/>
-        <v>single-input, single-output</v>
+        <f t="shared" ref="I41:I46" si="5">IF(E41="SIDO","single-input, double-output",IF(E41="SISO","single-input, single-output",IF(E41="PT","pass-through",IF(E41="DISO","double-input, single-output",IF(E41="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
+        <v>single-input, double-output</v>
       </c>
       <c r="J41" t="str">
-        <f t="shared" si="4"/>
-        <v>siso_methods</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.45">
+        <f t="shared" ref="J41:J46" si="6">IF(E41="SIDO","sido_methods",IF(E41="SISO","siso_methods",IF(E41="PT","pt_methods",IF(E41="DISO","diso_methods",IF(E41="SIDO reactive","sidor_methods","")))))</f>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B42" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C42" t="s">
-        <v>429</v>
+        <v>423</v>
       </c>
       <c r="D42" t="s">
         <v>30</v>
       </c>
       <c r="E42" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G42" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="H42" t="s">
-        <v>507</v>
+        <v>99</v>
       </c>
       <c r="I42" t="str">
-        <f t="shared" si="3"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="5"/>
+        <v>single-input, single-output</v>
       </c>
       <c r="J42" t="str">
-        <f t="shared" si="4"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.45">
+        <f t="shared" si="6"/>
+        <v>siso_methods</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B43" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C43" t="s">
-        <v>451</v>
+        <v>429</v>
       </c>
       <c r="D43" t="s">
         <v>30</v>
@@ -3449,69 +3424,69 @@
         <v>11</v>
       </c>
       <c r="F43" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G43" t="s">
-        <v>21</v>
-      </c>
-      <c r="H43" t="b">
-        <v>0</v>
+        <v>31</v>
+      </c>
+      <c r="H43" t="s">
+        <v>507</v>
       </c>
       <c r="I43" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J43" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>475</v>
+        <v>102</v>
       </c>
       <c r="B44" t="s">
-        <v>474</v>
+        <v>103</v>
       </c>
       <c r="C44" t="s">
-        <v>476</v>
+        <v>451</v>
       </c>
       <c r="D44" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E44" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F44" t="b">
         <v>1</v>
       </c>
       <c r="G44" t="s">
-        <v>12</v>
-      </c>
-      <c r="H44" t="s">
-        <v>477</v>
+        <v>21</v>
+      </c>
+      <c r="H44" t="b">
+        <v>0</v>
       </c>
       <c r="I44" t="str">
-        <f t="shared" si="3"/>
-        <v>reactive single-inlet, double-outlet</v>
+        <f t="shared" si="5"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J44" t="str">
-        <f t="shared" si="4"/>
-        <v>sidor_methods</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.45">
+        <f t="shared" si="6"/>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="B45" t="s">
-        <v>456</v>
+        <v>474</v>
       </c>
       <c r="C45" t="s">
-        <v>452</v>
+        <v>476</v>
       </c>
       <c r="D45" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E45" t="s">
         <v>18</v>
@@ -3520,64 +3495,63 @@
         <v>1</v>
       </c>
       <c r="G45" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="H45" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="I45" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>reactive single-inlet, double-outlet</v>
       </c>
       <c r="J45" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>sidor_methods</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>104</v>
+        <v>478</v>
       </c>
       <c r="B46" t="s">
-        <v>105</v>
+        <v>456</v>
       </c>
       <c r="C46" t="s">
-        <v>442</v>
+        <v>452</v>
       </c>
       <c r="D46" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E46" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="F46" t="b">
         <v>1</v>
       </c>
       <c r="G46" t="s">
-        <v>12</v>
-      </c>
-      <c r="H46" t="str">
-        <f>IF(D46="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+        <v>31</v>
+      </c>
+      <c r="H46" t="s">
+        <v>479</v>
       </c>
       <c r="I46" t="str">
-        <f t="shared" ref="I46:I92" si="5">IF(E46="SIDO","single-input, double-output",IF(E46="SISO","single-input, single-output",IF(E46="PT","pass-through",IF(E46="DISO","double-input, single-output",IF(E46="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
-        <v>pass-through</v>
+        <f t="shared" si="5"/>
+        <v>reactive single-inlet, double-outlet</v>
       </c>
       <c r="J46" t="str">
-        <f t="shared" ref="J46:J92" si="6">IF(E46="SIDO","sido_methods",IF(E46="SISO","siso_methods",IF(E46="PT","pt_methods",IF(E46="DISO","diso_methods",IF(E46="SIDO reactive","sidor_methods","")))))</f>
-        <v>pt_methods</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.45">
+        <f t="shared" si="6"/>
+        <v>sidor_methods</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B47" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C47" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="D47" t="s">
         <v>10</v>
@@ -3596,57 +3570,58 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I47" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="I47:I93" si="7">IF(E47="SIDO","single-input, double-output",IF(E47="SISO","single-input, single-output",IF(E47="PT","pass-through",IF(E47="DISO","double-input, single-output",IF(E47="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
         <v>pass-through</v>
       </c>
       <c r="J47" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="J47:J93" si="8">IF(E47="SIDO","sido_methods",IF(E47="SISO","siso_methods",IF(E47="PT","pt_methods",IF(E47="DISO","diso_methods",IF(E47="SIDO reactive","sidor_methods","")))))</f>
         <v>pt_methods</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B48" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C48" t="s">
-        <v>427</v>
+        <v>441</v>
       </c>
       <c r="D48" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E48" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F48" t="b">
         <v>1</v>
       </c>
       <c r="G48" t="s">
-        <v>21</v>
-      </c>
-      <c r="H48" t="s">
-        <v>110</v>
+        <v>12</v>
+      </c>
+      <c r="H48" t="str">
+        <f>IF(D48="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I48" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="7"/>
+        <v>pass-through</v>
       </c>
       <c r="J48" t="str">
-        <f t="shared" si="6"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.45">
+        <f t="shared" si="8"/>
+        <v>pt_methods</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B49" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C49" t="s">
-        <v>397</v>
+        <v>427</v>
       </c>
       <c r="D49" t="s">
         <v>30</v>
@@ -3655,72 +3630,72 @@
         <v>11</v>
       </c>
       <c r="F49" t="b">
+        <v>1</v>
+      </c>
+      <c r="G49" t="s">
+        <v>21</v>
+      </c>
+      <c r="H49" t="s">
+        <v>110</v>
+      </c>
+      <c r="I49" t="str">
+        <f t="shared" si="7"/>
+        <v>single-input, double-output</v>
+      </c>
+      <c r="J49" t="str">
+        <f t="shared" si="8"/>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>111</v>
+      </c>
+      <c r="B50" t="s">
+        <v>112</v>
+      </c>
+      <c r="C50" t="s">
+        <v>397</v>
+      </c>
+      <c r="D50" t="s">
+        <v>30</v>
+      </c>
+      <c r="E50" t="s">
+        <v>11</v>
+      </c>
+      <c r="F50" t="b">
         <v>0</v>
       </c>
-      <c r="G49" t="s">
+      <c r="G50" t="s">
         <v>31</v>
       </c>
-      <c r="H49" t="s">
+      <c r="H50" t="s">
         <v>113</v>
       </c>
-      <c r="I49" t="str">
-        <f t="shared" si="5"/>
+      <c r="I50" t="str">
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
-      <c r="J49" t="str">
-        <f t="shared" si="6"/>
+      <c r="J50" t="str">
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A50" t="s">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
         <v>114</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B51" t="s">
         <v>115</v>
       </c>
-      <c r="C50" t="s">
+      <c r="C51" t="s">
         <v>398</v>
       </c>
-      <c r="D50" t="s">
+      <c r="D51" t="s">
         <v>10</v>
       </c>
-      <c r="E50" t="s">
+      <c r="E51" t="s">
         <v>27</v>
-      </c>
-      <c r="F50" t="b">
-        <v>1</v>
-      </c>
-      <c r="G50" t="s">
-        <v>12</v>
-      </c>
-      <c r="H50" t="s">
-        <v>116</v>
-      </c>
-      <c r="I50" t="str">
-        <f t="shared" si="5"/>
-        <v>pass-through</v>
-      </c>
-      <c r="J50" t="str">
-        <f t="shared" si="6"/>
-        <v>pt_methods</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A51" t="s">
-        <v>117</v>
-      </c>
-      <c r="B51" t="s">
-        <v>118</v>
-      </c>
-      <c r="C51" t="s">
-        <v>400</v>
-      </c>
-      <c r="D51" t="s">
-        <v>30</v>
-      </c>
-      <c r="E51" t="s">
-        <v>18</v>
       </c>
       <c r="F51" t="b">
         <v>1</v>
@@ -3729,26 +3704,26 @@
         <v>12</v>
       </c>
       <c r="H51" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="I51" t="str">
-        <f t="shared" si="5"/>
-        <v>reactive single-inlet, double-outlet</v>
+        <f t="shared" si="7"/>
+        <v>pass-through</v>
       </c>
       <c r="J51" t="str">
-        <f t="shared" si="6"/>
-        <v>sidor_methods</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.45">
+        <f t="shared" si="8"/>
+        <v>pt_methods</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>480</v>
+        <v>117</v>
       </c>
       <c r="B52" t="s">
-        <v>481</v>
+        <v>118</v>
       </c>
       <c r="C52" t="s">
-        <v>482</v>
+        <v>400</v>
       </c>
       <c r="D52" t="s">
         <v>30</v>
@@ -3763,32 +3738,32 @@
         <v>12</v>
       </c>
       <c r="H52" t="s">
-        <v>483</v>
+        <v>119</v>
       </c>
       <c r="I52" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>reactive single-inlet, double-outlet</v>
       </c>
       <c r="J52" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sidor_methods</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>120</v>
+        <v>480</v>
       </c>
       <c r="B53" t="s">
-        <v>121</v>
+        <v>481</v>
       </c>
       <c r="C53" t="s">
-        <v>401</v>
+        <v>482</v>
       </c>
       <c r="D53" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E53" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F53" t="b">
         <v>1</v>
@@ -3796,28 +3771,27 @@
       <c r="G53" t="s">
         <v>12</v>
       </c>
-      <c r="H53" t="str">
-        <f>IF(D53="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H53" t="s">
+        <v>483</v>
       </c>
       <c r="I53" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="7"/>
+        <v>reactive single-inlet, double-outlet</v>
       </c>
       <c r="J53" t="str">
-        <f t="shared" si="6"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.45">
+        <f t="shared" si="8"/>
+        <v>sidor_methods</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B54" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C54" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="D54" t="s">
         <v>10</v>
@@ -3836,26 +3810,26 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I54" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J54" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>484</v>
+        <v>122</v>
       </c>
       <c r="B55" t="s">
-        <v>485</v>
+        <v>123</v>
       </c>
       <c r="C55" t="s">
-        <v>486</v>
+        <v>402</v>
       </c>
       <c r="D55" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E55" t="s">
         <v>11</v>
@@ -3866,61 +3840,62 @@
       <c r="G55" t="s">
         <v>12</v>
       </c>
-      <c r="H55" t="s">
-        <v>487</v>
+      <c r="H55" t="str">
+        <f>IF(D55="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I55" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J55" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>124</v>
+        <v>484</v>
       </c>
       <c r="B56" t="s">
-        <v>125</v>
+        <v>485</v>
       </c>
       <c r="C56" t="s">
-        <v>386</v>
+        <v>486</v>
       </c>
       <c r="D56" t="s">
         <v>30</v>
       </c>
       <c r="E56" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F56" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G56" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="H56" t="s">
-        <v>126</v>
+        <v>487</v>
       </c>
       <c r="I56" t="str">
-        <f t="shared" si="5"/>
-        <v>reactive single-inlet, double-outlet</v>
+        <f t="shared" si="7"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J56" t="str">
-        <f t="shared" si="6"/>
-        <v>sidor_methods</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.45">
+        <f t="shared" si="8"/>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>488</v>
+        <v>124</v>
       </c>
       <c r="B57" t="s">
-        <v>489</v>
+        <v>125</v>
       </c>
       <c r="C57" t="s">
-        <v>490</v>
+        <v>386</v>
       </c>
       <c r="D57" t="s">
         <v>30</v>
@@ -3929,38 +3904,38 @@
         <v>18</v>
       </c>
       <c r="F57" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G57" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="H57" t="s">
-        <v>491</v>
+        <v>126</v>
       </c>
       <c r="I57" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>reactive single-inlet, double-outlet</v>
       </c>
       <c r="J57" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sidor_methods</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>127</v>
+        <v>488</v>
       </c>
       <c r="B58" t="s">
-        <v>128</v>
+        <v>489</v>
       </c>
       <c r="C58" t="s">
-        <v>403</v>
+        <v>490</v>
       </c>
       <c r="D58" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E58" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F58" t="b">
         <v>1</v>
@@ -3968,28 +3943,27 @@
       <c r="G58" t="s">
         <v>12</v>
       </c>
-      <c r="H58" t="str">
-        <f>IF(D58="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H58" t="s">
+        <v>491</v>
       </c>
       <c r="I58" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="7"/>
+        <v>reactive single-inlet, double-outlet</v>
       </c>
       <c r="J58" t="str">
-        <f t="shared" si="6"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.45">
+        <f t="shared" si="8"/>
+        <v>sidor_methods</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B59" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C59" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="D59" t="s">
         <v>10</v>
@@ -4008,57 +3982,58 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I59" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J59" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B60" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C60" t="s">
-        <v>424</v>
+        <v>404</v>
       </c>
       <c r="D60" t="s">
         <v>10</v>
       </c>
       <c r="E60" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F60" t="b">
         <v>1</v>
       </c>
       <c r="G60" t="s">
-        <v>21</v>
-      </c>
-      <c r="H60" t="s">
-        <v>65</v>
+        <v>12</v>
+      </c>
+      <c r="H60" t="str">
+        <f>IF(D60="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I60" t="str">
-        <f t="shared" si="5"/>
-        <v>pass-through</v>
+        <f t="shared" si="7"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J60" t="str">
-        <f t="shared" si="6"/>
-        <v>pt_methods</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.45">
+        <f t="shared" si="8"/>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B61" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C61" t="s">
-        <v>405</v>
+        <v>424</v>
       </c>
       <c r="D61" t="s">
         <v>10</v>
@@ -4070,70 +4045,70 @@
         <v>1</v>
       </c>
       <c r="G61" t="s">
+        <v>21</v>
+      </c>
+      <c r="H61" t="s">
+        <v>65</v>
+      </c>
+      <c r="I61" t="str">
+        <f t="shared" si="7"/>
+        <v>pass-through</v>
+      </c>
+      <c r="J61" t="str">
+        <f t="shared" si="8"/>
+        <v>pt_methods</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>133</v>
+      </c>
+      <c r="B62" t="s">
+        <v>134</v>
+      </c>
+      <c r="C62" t="s">
+        <v>405</v>
+      </c>
+      <c r="D62" t="s">
+        <v>10</v>
+      </c>
+      <c r="E62" t="s">
+        <v>27</v>
+      </c>
+      <c r="F62" t="b">
+        <v>1</v>
+      </c>
+      <c r="G62" t="s">
         <v>12</v>
       </c>
-      <c r="H61" t="str">
-        <f>IF(D61="basic","cost_power_law_flow")</f>
+      <c r="H62" t="str">
+        <f>IF(D62="basic","cost_power_law_flow")</f>
         <v>cost_power_law_flow</v>
       </c>
-      <c r="I61" t="str">
-        <f t="shared" si="5"/>
+      <c r="I62" t="str">
+        <f t="shared" si="7"/>
         <v>pass-through</v>
       </c>
-      <c r="J61" t="str">
-        <f t="shared" si="6"/>
+      <c r="J62" t="str">
+        <f t="shared" si="8"/>
         <v>pt_methods</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A62" t="s">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
         <v>135</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B63" t="s">
         <v>136</v>
       </c>
-      <c r="C62" t="s">
+      <c r="C63" t="s">
         <v>406</v>
-      </c>
-      <c r="D62" t="s">
-        <v>30</v>
-      </c>
-      <c r="E62" t="s">
-        <v>11</v>
-      </c>
-      <c r="F62" t="b">
-        <v>0</v>
-      </c>
-      <c r="G62" t="s">
-        <v>31</v>
-      </c>
-      <c r="H62" t="s">
-        <v>137</v>
-      </c>
-      <c r="I62" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, double-output</v>
-      </c>
-      <c r="J62" t="str">
-        <f t="shared" si="6"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A63" t="s">
-        <v>138</v>
-      </c>
-      <c r="B63" t="s">
-        <v>370</v>
-      </c>
-      <c r="C63" t="s">
-        <v>426</v>
       </c>
       <c r="D63" t="s">
         <v>30</v>
       </c>
       <c r="E63" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F63" t="b">
         <v>0</v>
@@ -4142,26 +4117,26 @@
         <v>31</v>
       </c>
       <c r="H63" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I63" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, single-output</v>
+        <f t="shared" si="7"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J63" t="str">
-        <f t="shared" si="6"/>
-        <v>siso_methods</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.45">
+        <f t="shared" si="8"/>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B64" t="s">
-        <v>141</v>
+        <v>370</v>
       </c>
       <c r="C64" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D64" t="s">
         <v>30</v>
@@ -4176,204 +4151,203 @@
         <v>31</v>
       </c>
       <c r="H64" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="I64" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, single-output</v>
       </c>
       <c r="J64" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>siso_methods</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>492</v>
+        <v>140</v>
       </c>
       <c r="B65" t="s">
-        <v>493</v>
+        <v>141</v>
       </c>
       <c r="C65" t="s">
-        <v>494</v>
+        <v>425</v>
       </c>
       <c r="D65" t="s">
         <v>30</v>
       </c>
       <c r="E65" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="F65" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G65" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="H65" t="s">
-        <v>495</v>
+        <v>142</v>
       </c>
       <c r="I65" t="str">
-        <f t="shared" si="5"/>
-        <v>reactive single-inlet, double-outlet</v>
+        <f t="shared" si="7"/>
+        <v>single-input, single-output</v>
       </c>
       <c r="J65" t="str">
-        <f t="shared" si="6"/>
-        <v>sidor_methods</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.45">
+        <f t="shared" si="8"/>
+        <v>siso_methods</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>143</v>
+        <v>492</v>
       </c>
       <c r="B66" t="s">
-        <v>144</v>
+        <v>493</v>
       </c>
       <c r="C66" t="s">
-        <v>444</v>
+        <v>494</v>
       </c>
       <c r="D66" t="s">
         <v>30</v>
       </c>
       <c r="E66" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F66" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G66" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="H66" t="s">
-        <v>145</v>
+        <v>495</v>
       </c>
       <c r="I66" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="7"/>
+        <v>reactive single-inlet, double-outlet</v>
       </c>
       <c r="J66" t="str">
-        <f t="shared" si="6"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.45">
+        <f t="shared" si="8"/>
+        <v>sidor_methods</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B67" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C67" t="s">
-        <v>408</v>
+        <v>444</v>
       </c>
       <c r="D67" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E67" t="s">
         <v>11</v>
       </c>
       <c r="F67" t="b">
+        <v>0</v>
+      </c>
+      <c r="G67" t="s">
+        <v>31</v>
+      </c>
+      <c r="H67" t="s">
+        <v>145</v>
+      </c>
+      <c r="I67" t="str">
+        <f t="shared" si="7"/>
+        <v>single-input, double-output</v>
+      </c>
+      <c r="J67" t="str">
+        <f t="shared" si="8"/>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>146</v>
+      </c>
+      <c r="B68" t="s">
+        <v>147</v>
+      </c>
+      <c r="C68" t="s">
+        <v>408</v>
+      </c>
+      <c r="D68" t="s">
+        <v>10</v>
+      </c>
+      <c r="E68" t="s">
+        <v>11</v>
+      </c>
+      <c r="F68" t="b">
         <v>1</v>
       </c>
-      <c r="G67" t="s">
+      <c r="G68" t="s">
         <v>12</v>
       </c>
-      <c r="H67" t="str">
-        <f>IF(D67="basic","cost_power_law_flow")</f>
+      <c r="H68" t="str">
+        <f>IF(D68="basic","cost_power_law_flow")</f>
         <v>cost_power_law_flow</v>
       </c>
-      <c r="I67" t="str">
-        <f t="shared" si="5"/>
+      <c r="I68" t="str">
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
-      <c r="J67" t="str">
-        <f t="shared" si="6"/>
+      <c r="J68" t="str">
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A68" t="s">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
         <v>148</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B69" t="s">
         <v>149</v>
       </c>
-      <c r="C68" t="s">
+      <c r="C69" t="s">
         <v>399</v>
       </c>
-      <c r="D68" t="s">
+      <c r="D69" t="s">
         <v>30</v>
-      </c>
-      <c r="E68" t="s">
-        <v>27</v>
-      </c>
-      <c r="F68" t="b">
-        <v>0</v>
-      </c>
-      <c r="G68" t="s">
-        <v>31</v>
-      </c>
-      <c r="H68" t="s">
-        <v>150</v>
-      </c>
-      <c r="I68" t="str">
-        <f t="shared" si="5"/>
-        <v>pass-through</v>
-      </c>
-      <c r="J68" t="str">
-        <f t="shared" si="6"/>
-        <v>pt_methods</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A69" t="s">
-        <v>151</v>
-      </c>
-      <c r="B69" t="s">
-        <v>152</v>
-      </c>
-      <c r="C69" t="s">
-        <v>409</v>
-      </c>
-      <c r="D69" t="s">
-        <v>10</v>
       </c>
       <c r="E69" t="s">
         <v>27</v>
       </c>
       <c r="F69" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G69" t="s">
-        <v>12</v>
-      </c>
-      <c r="H69" t="str">
-        <f>IF(D69="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+        <v>31</v>
+      </c>
+      <c r="H69" t="s">
+        <v>150</v>
       </c>
       <c r="I69" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>pass-through</v>
       </c>
       <c r="J69" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>pt_methods</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B70" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C70" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="D70" t="s">
         <v>10</v>
       </c>
       <c r="E70" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F70" t="b">
         <v>1</v>
@@ -4386,26 +4360,26 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I70" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="7"/>
+        <v>pass-through</v>
       </c>
       <c r="J70" t="str">
-        <f t="shared" si="6"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.45">
+        <f t="shared" si="8"/>
+        <v>pt_methods</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B71" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C71" t="s">
-        <v>448</v>
+        <v>410</v>
       </c>
       <c r="D71" t="s">
-        <v>57</v>
+        <v>10</v>
       </c>
       <c r="E71" t="s">
         <v>11</v>
@@ -4416,30 +4390,31 @@
       <c r="G71" t="s">
         <v>12</v>
       </c>
-      <c r="H71" t="s">
-        <v>65</v>
+      <c r="H71" t="str">
+        <f>IF(D71="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I71" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J71" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B72" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C72" t="s">
-        <v>411</v>
+        <v>448</v>
       </c>
       <c r="D72" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="E72" t="s">
         <v>11</v>
@@ -4451,29 +4426,29 @@
         <v>12</v>
       </c>
       <c r="H72" t="s">
-        <v>159</v>
+        <v>65</v>
       </c>
       <c r="I72" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J72" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B73" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="D73" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E73" t="s">
         <v>11</v>
@@ -4484,28 +4459,27 @@
       <c r="G73" t="s">
         <v>12</v>
       </c>
-      <c r="H73" t="str">
-        <f>IF(D73="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H73" t="s">
+        <v>159</v>
       </c>
       <c r="I73" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J73" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B74" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C74" t="s">
-        <v>436</v>
+        <v>412</v>
       </c>
       <c r="D74" t="s">
         <v>10</v>
@@ -4524,29 +4498,29 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I74" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J74" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B75" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C75" t="s">
-        <v>413</v>
+        <v>436</v>
       </c>
       <c r="D75" t="s">
         <v>10</v>
       </c>
       <c r="E75" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F75" t="b">
         <v>1</v>
@@ -4559,23 +4533,23 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I75" t="str">
-        <f t="shared" si="5"/>
-        <v>pass-through</v>
+        <f t="shared" si="7"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J75" t="str">
-        <f t="shared" si="6"/>
-        <v>pt_methods</v>
-      </c>
-    </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.45">
+        <f t="shared" si="8"/>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B76" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C76" t="s">
-        <v>434</v>
+        <v>413</v>
       </c>
       <c r="D76" t="s">
         <v>10</v>
@@ -4594,26 +4568,26 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I76" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>pass-through</v>
       </c>
       <c r="J76" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>pt_methods</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B77" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C77" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="D77" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E77" t="s">
         <v>27</v>
@@ -4624,30 +4598,31 @@
       <c r="G77" t="s">
         <v>12</v>
       </c>
-      <c r="H77" t="s">
-        <v>170</v>
+      <c r="H77" t="str">
+        <f>IF(D77="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I77" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>pass-through</v>
       </c>
       <c r="J77" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>pt_methods</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>496</v>
+        <v>168</v>
       </c>
       <c r="B78" t="s">
-        <v>497</v>
+        <v>169</v>
       </c>
       <c r="C78" t="s">
-        <v>498</v>
+        <v>431</v>
       </c>
       <c r="D78" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E78" t="s">
         <v>27</v>
@@ -4659,32 +4634,32 @@
         <v>12</v>
       </c>
       <c r="H78" t="s">
-        <v>499</v>
+        <v>170</v>
       </c>
       <c r="I78" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>pass-through</v>
       </c>
       <c r="J78" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>pt_methods</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="B79" t="s">
-        <v>501</v>
+        <v>497</v>
       </c>
       <c r="C79" t="s">
-        <v>502</v>
+        <v>498</v>
       </c>
       <c r="D79" t="s">
         <v>10</v>
       </c>
       <c r="E79" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F79" t="b">
         <v>1</v>
@@ -4693,97 +4668,97 @@
         <v>12</v>
       </c>
       <c r="H79" t="s">
-        <v>503</v>
+        <v>499</v>
       </c>
       <c r="I79" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="7"/>
+        <v>pass-through</v>
       </c>
       <c r="J79" t="str">
-        <f t="shared" si="6"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.45">
+        <f t="shared" si="8"/>
+        <v>pt_methods</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>504</v>
+        <v>500</v>
       </c>
       <c r="B80" t="s">
-        <v>457</v>
+        <v>501</v>
       </c>
       <c r="C80" t="s">
-        <v>453</v>
+        <v>502</v>
       </c>
       <c r="D80" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E80" t="s">
         <v>11</v>
       </c>
       <c r="F80" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G80" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="H80" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="I80" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J80" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>171</v>
+        <v>504</v>
       </c>
       <c r="B81" t="s">
-        <v>172</v>
+        <v>457</v>
       </c>
       <c r="C81" t="s">
-        <v>443</v>
+        <v>453</v>
       </c>
       <c r="D81" t="s">
         <v>30</v>
       </c>
       <c r="E81" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F81" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G81" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="H81" t="s">
-        <v>173</v>
+        <v>505</v>
       </c>
       <c r="I81" t="str">
-        <f t="shared" si="5"/>
-        <v>pass-through</v>
+        <f t="shared" si="7"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J81" t="str">
-        <f t="shared" si="6"/>
-        <v>pt_methods</v>
-      </c>
-    </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.45">
+        <f t="shared" si="8"/>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="B82" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C82" t="s">
-        <v>432</v>
+        <v>443</v>
       </c>
       <c r="D82" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E82" t="s">
         <v>27</v>
@@ -4794,28 +4769,27 @@
       <c r="G82" t="s">
         <v>21</v>
       </c>
-      <c r="H82" t="str">
-        <f>IF(D82="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H82" t="s">
+        <v>173</v>
       </c>
       <c r="I82" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>pass-through</v>
       </c>
       <c r="J82" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>pt_methods</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B83" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C83" t="s">
-        <v>414</v>
+        <v>432</v>
       </c>
       <c r="D83" t="s">
         <v>10</v>
@@ -4827,36 +4801,36 @@
         <v>1</v>
       </c>
       <c r="G83" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="H83" t="str">
         <f>IF(D83="basic","cost_power_law_flow")</f>
         <v>cost_power_law_flow</v>
       </c>
       <c r="I83" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>pass-through</v>
       </c>
       <c r="J83" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>pt_methods</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B84" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C84" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="D84" t="s">
         <v>10</v>
       </c>
       <c r="E84" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F84" t="b">
         <v>1</v>
@@ -4869,23 +4843,23 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I84" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="7"/>
+        <v>pass-through</v>
       </c>
       <c r="J84" t="str">
-        <f t="shared" si="6"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.45">
+        <f t="shared" si="8"/>
+        <v>pt_methods</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B85" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C85" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D85" t="s">
         <v>10</v>
@@ -4904,29 +4878,29 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I85" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J85" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B86" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C86" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="D86" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E86" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F86" t="b">
         <v>1</v>
@@ -4934,27 +4908,28 @@
       <c r="G86" t="s">
         <v>12</v>
       </c>
-      <c r="H86" t="s">
-        <v>184</v>
+      <c r="H86" t="str">
+        <f>IF(D86="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I86" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, single-output</v>
+        <f t="shared" si="7"/>
+        <v>single-input, double-output</v>
       </c>
       <c r="J86" t="str">
-        <f t="shared" si="6"/>
-        <v>siso_methods</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.45">
+        <f t="shared" si="8"/>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="B87" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C87" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D87" t="s">
         <v>30</v>
@@ -4969,32 +4944,32 @@
         <v>12</v>
       </c>
       <c r="H87" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="I87" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, single-output</v>
       </c>
       <c r="J87" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>siso_methods</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B88" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C88" t="s">
-        <v>454</v>
+        <v>418</v>
       </c>
       <c r="D88" t="s">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="E88" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F88" t="b">
         <v>1</v>
@@ -5003,29 +4978,29 @@
         <v>12</v>
       </c>
       <c r="H88" t="s">
-        <v>461</v>
+        <v>187</v>
       </c>
       <c r="I88" t="str">
-        <f t="shared" si="5"/>
-        <v>single-input, double-output</v>
+        <f t="shared" si="7"/>
+        <v>single-input, single-output</v>
       </c>
       <c r="J88" t="str">
-        <f t="shared" si="6"/>
-        <v>sido_methods</v>
-      </c>
-    </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.45">
+        <f t="shared" si="8"/>
+        <v>siso_methods</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B89" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C89" t="s">
-        <v>421</v>
+        <v>454</v>
       </c>
       <c r="D89" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="E89" t="s">
         <v>11</v>
@@ -5036,28 +5011,27 @@
       <c r="G89" t="s">
         <v>12</v>
       </c>
-      <c r="H89" t="str">
-        <f>IF(D89="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H89" t="s">
+        <v>461</v>
       </c>
       <c r="I89" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J89" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B90" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C90" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D90" t="s">
         <v>10</v>
@@ -5076,57 +5050,58 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I90" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>single-input, double-output</v>
       </c>
       <c r="J90" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>sido_methods</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
+        <v>192</v>
+      </c>
+      <c r="B91" t="s">
+        <v>193</v>
+      </c>
+      <c r="C91" t="s">
+        <v>420</v>
+      </c>
+      <c r="D91" t="s">
+        <v>10</v>
+      </c>
+      <c r="E91" t="s">
+        <v>11</v>
+      </c>
+      <c r="F91" t="b">
+        <v>1</v>
+      </c>
+      <c r="G91" t="s">
+        <v>12</v>
+      </c>
+      <c r="H91" t="str">
+        <f>IF(D91="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
+      </c>
+      <c r="I91" t="str">
+        <f t="shared" si="7"/>
+        <v>single-input, double-output</v>
+      </c>
+      <c r="J91" t="str">
+        <f t="shared" si="8"/>
+        <v>sido_methods</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
         <v>194</v>
       </c>
-      <c r="B91" t="s">
+      <c r="B92" t="s">
         <v>195</v>
       </c>
-      <c r="C91" t="s">
+      <c r="C92" t="s">
         <v>439</v>
-      </c>
-      <c r="D91" t="s">
-        <v>30</v>
-      </c>
-      <c r="E91" t="s">
-        <v>27</v>
-      </c>
-      <c r="F91" t="b">
-        <v>0</v>
-      </c>
-      <c r="G91" t="s">
-        <v>31</v>
-      </c>
-      <c r="H91" t="s">
-        <v>65</v>
-      </c>
-      <c r="I91" t="str">
-        <f t="shared" si="5"/>
-        <v>pass-through</v>
-      </c>
-      <c r="J91" t="str">
-        <f t="shared" si="6"/>
-        <v>pt_methods</v>
-      </c>
-    </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="A92" t="s">
-        <v>196</v>
-      </c>
-      <c r="B92" t="s">
-        <v>197</v>
-      </c>
-      <c r="C92" t="s">
-        <v>440</v>
       </c>
       <c r="D92" t="s">
         <v>30</v>
@@ -5135,26 +5110,60 @@
         <v>27</v>
       </c>
       <c r="F92" t="b">
+        <v>0</v>
+      </c>
+      <c r="G92" t="s">
+        <v>31</v>
+      </c>
+      <c r="H92" t="s">
+        <v>65</v>
+      </c>
+      <c r="I92" t="str">
+        <f t="shared" si="7"/>
+        <v>pass-through</v>
+      </c>
+      <c r="J92" t="str">
+        <f t="shared" si="8"/>
+        <v>pt_methods</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>196</v>
+      </c>
+      <c r="B93" t="s">
+        <v>197</v>
+      </c>
+      <c r="C93" t="s">
+        <v>440</v>
+      </c>
+      <c r="D93" t="s">
+        <v>30</v>
+      </c>
+      <c r="E93" t="s">
+        <v>27</v>
+      </c>
+      <c r="F93" t="b">
         <v>1</v>
       </c>
-      <c r="G92" t="s">
+      <c r="G93" t="s">
         <v>21</v>
       </c>
-      <c r="H92" t="s">
+      <c r="H93" t="s">
         <v>198</v>
       </c>
-      <c r="I92" t="str">
-        <f t="shared" si="5"/>
+      <c r="I93" t="str">
+        <f t="shared" si="7"/>
         <v>pass-through</v>
       </c>
-      <c r="J92" t="str">
-        <f t="shared" si="6"/>
+      <c r="J93" t="str">
+        <f t="shared" si="8"/>
         <v>pt_methods</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J92">
-    <sortCondition ref="B2:B92"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J93">
+    <sortCondition ref="B2:B93"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -5164,14 +5173,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G77"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
-    <col min="2" max="2" width="33.53125" customWidth="1"/>
-    <col min="3" max="3" width="31.46484375" customWidth="1"/>
+    <col min="2" max="2" width="33.5" customWidth="1"/>
+    <col min="3" max="3" width="31.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>199</v>
       </c>
@@ -5190,7 +5199,7 @@
         <v>aeration basin</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>202</v>
       </c>
@@ -5209,7 +5218,7 @@
         <v>air flotation</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>205</v>
       </c>
@@ -5231,7 +5240,7 @@
         <v>anaerobic digestion</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>209</v>
       </c>
@@ -5253,7 +5262,7 @@
         <v>anaerobic mbr mec</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>212</v>
       </c>
@@ -5275,7 +5284,7 @@
         <v>backwash solids handling</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>216</v>
       </c>
@@ -5297,7 +5306,7 @@
         <v>bio active filtration</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>220</v>
       </c>
@@ -5313,7 +5322,7 @@
         <v xml:space="preserve">bioreactor </v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>221</v>
       </c>
@@ -5332,7 +5341,7 @@
         <v>blending resevoir</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>224</v>
       </c>
@@ -5351,7 +5360,7 @@
         <v>brine concentrator</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>227</v>
       </c>
@@ -5370,7 +5379,7 @@
         <v>buffer tank</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>230</v>
       </c>
@@ -5386,7 +5395,7 @@
         <v xml:space="preserve">CANDOP </v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>231</v>
       </c>
@@ -5405,7 +5414,7 @@
         <v>cartridge filtration</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>233</v>
       </c>
@@ -5424,7 +5433,7 @@
         <v>chemical addition</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>236</v>
       </c>
@@ -5440,7 +5449,7 @@
         <v xml:space="preserve">chlorination </v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>237</v>
       </c>
@@ -5456,7 +5465,7 @@
         <v xml:space="preserve">clarifier </v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>238</v>
       </c>
@@ -5475,7 +5484,7 @@
         <v>co2 addition</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>240</v>
       </c>
@@ -5497,7 +5506,7 @@
         <v>coag and floc</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>244</v>
       </c>
@@ -5513,7 +5522,7 @@
         <v xml:space="preserve">cofermentation  </v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>245</v>
       </c>
@@ -5532,7 +5541,7 @@
         <v xml:space="preserve">constructed wetlands </v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>248</v>
       </c>
@@ -5554,7 +5563,7 @@
         <v>conventional activated sludge</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>252</v>
       </c>
@@ -5573,7 +5582,7 @@
         <v xml:space="preserve">cooling supply </v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>255</v>
       </c>
@@ -5592,7 +5601,7 @@
         <v xml:space="preserve">cooling tower </v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>257</v>
       </c>
@@ -5608,7 +5617,7 @@
         <v xml:space="preserve">decarbonator </v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>258</v>
       </c>
@@ -5630,7 +5639,7 @@
         <v>deep well injection</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>262</v>
       </c>
@@ -5652,7 +5661,7 @@
         <v>dissolved air flotation</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>264</v>
       </c>
@@ -5668,7 +5677,7 @@
         <v xml:space="preserve">dmbr </v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>265</v>
       </c>
@@ -5690,7 +5699,7 @@
         <v>dual media filtration</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>268</v>
       </c>
@@ -5712,7 +5721,7 @@
         <v>electrochemical nutrient removal</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>272</v>
       </c>
@@ -5731,7 +5740,7 @@
         <v>electrodialysis reversal</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>275</v>
       </c>
@@ -5750,7 +5759,7 @@
         <v>energy recovery</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>277</v>
       </c>
@@ -5769,7 +5778,7 @@
         <v>evaporation pond</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>280</v>
       </c>
@@ -5791,7 +5800,7 @@
         <v>feed water tank</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>281</v>
       </c>
@@ -5807,7 +5816,7 @@
         <v xml:space="preserve">feed </v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>283</v>
       </c>
@@ -5826,7 +5835,7 @@
         <v>filter press</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>286</v>
       </c>
@@ -5845,7 +5854,7 @@
         <v>fixed bed</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>289</v>
       </c>
@@ -5861,7 +5870,7 @@
         <v xml:space="preserve">gac </v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>290</v>
       </c>
@@ -5883,7 +5892,7 @@
         <v>gas sparged membrane</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>294</v>
       </c>
@@ -5905,7 +5914,7 @@
         <v>injection well disposal</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>296</v>
       </c>
@@ -5924,7 +5933,7 @@
         <v>intrusion mitigation</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>299</v>
       </c>
@@ -5943,7 +5952,7 @@
         <v>ion exchange</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>302</v>
       </c>
@@ -5968,7 +5977,7 @@
         <v>iron and manganese removal</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>305</v>
       </c>
@@ -5984,7 +5993,7 @@
         <v xml:space="preserve">landfill </v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>306</v>
       </c>
@@ -6000,7 +6009,7 @@
         <v xml:space="preserve">mabr </v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>210</v>
       </c>
@@ -6016,7 +6025,7 @@
         <v xml:space="preserve">mbr </v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>307</v>
       </c>
@@ -6035,7 +6044,7 @@
         <v>media filtration</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>308</v>
       </c>
@@ -6051,7 +6060,7 @@
         <v xml:space="preserve">metab </v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>309</v>
       </c>
@@ -6067,7 +6076,7 @@
         <v xml:space="preserve">microfiltration </v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>310</v>
       </c>
@@ -6086,7 +6095,7 @@
         <v>microscreen filtration</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>312</v>
       </c>
@@ -6105,7 +6114,7 @@
         <v>municipal drinking</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>315</v>
       </c>
@@ -6124,7 +6133,7 @@
         <v>municipal wwtp</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>317</v>
       </c>
@@ -6140,7 +6149,7 @@
         <v xml:space="preserve">nanofiltration </v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>318</v>
       </c>
@@ -6159,7 +6168,7 @@
         <v xml:space="preserve">ozone aop </v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
         <v>319</v>
       </c>
@@ -6175,7 +6184,7 @@
         <v xml:space="preserve">ozone </v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
         <v>321</v>
       </c>
@@ -6194,7 +6203,7 @@
         <v>photothermal membrane</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>323</v>
       </c>
@@ -6213,7 +6222,7 @@
         <v>primary separator</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
         <v>21</v>
       </c>
@@ -6232,7 +6241,7 @@
         <v>pump electricity</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
         <v>326</v>
       </c>
@@ -6248,7 +6257,7 @@
         <v xml:space="preserve">pump </v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>328</v>
       </c>
@@ -6264,7 +6273,7 @@
         <v xml:space="preserve">screen </v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>329</v>
       </c>
@@ -6286,7 +6295,7 @@
         <v>secondary treatment wwtp</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
         <v>332</v>
       </c>
@@ -6302,7 +6311,7 @@
         <v xml:space="preserve">sedimentation </v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
         <v>333</v>
       </c>
@@ -6321,7 +6330,7 @@
         <v>settling pond</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
         <v>335</v>
       </c>
@@ -6340,7 +6349,7 @@
         <v>sludge tank</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
         <v>336</v>
       </c>
@@ -6356,7 +6365,7 @@
         <v xml:space="preserve">smp </v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
         <v>337</v>
       </c>
@@ -6375,7 +6384,7 @@
         <v>static mixer</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
         <v>340</v>
       </c>
@@ -6394,7 +6403,7 @@
         <v>storage tank</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>342</v>
       </c>
@@ -6413,7 +6422,7 @@
         <v>surface discharge</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
         <v>345</v>
       </c>
@@ -6435,7 +6444,7 @@
         <v>sw onshore intake</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
         <v>349</v>
       </c>
@@ -6457,7 +6466,7 @@
         <v>tramp oil tank</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
         <v>352</v>
       </c>
@@ -6479,7 +6488,7 @@
         <v>tri media filtration</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
         <v>354</v>
       </c>
@@ -6498,7 +6507,7 @@
         <v>ultra filtration</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
         <v>356</v>
       </c>
@@ -6517,7 +6526,7 @@
         <v>uv aop</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
         <v>357</v>
       </c>
@@ -6533,7 +6542,7 @@
         <v xml:space="preserve">uv </v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
         <v>359</v>
       </c>
@@ -6552,7 +6561,7 @@
         <v>vfa recovery</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
         <v>361</v>
       </c>
@@ -6568,7 +6577,7 @@
         <v xml:space="preserve">waiv </v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
         <v>362</v>
       </c>
@@ -6590,7 +6599,7 @@
         <v>walnut shell filter</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
         <v>365</v>
       </c>
@@ -6612,7 +6621,7 @@
         <v>water pumping station</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
         <v>368</v>
       </c>
@@ -6640,12 +6649,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B1:C80"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="37.19921875" customWidth="1"/>
+    <col min="2" max="2" width="37.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>9</v>
       </c>
@@ -6653,7 +6662,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>14</v>
       </c>
@@ -6661,7 +6670,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>15</v>
       </c>
@@ -6669,7 +6678,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>17</v>
       </c>
@@ -6677,7 +6686,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>455</v>
       </c>
@@ -6685,7 +6694,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>20</v>
       </c>
@@ -6693,7 +6702,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>23</v>
       </c>
@@ -6701,7 +6710,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
         <v>25</v>
       </c>
@@ -6709,7 +6718,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
         <v>371</v>
       </c>
@@ -6717,7 +6726,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>29</v>
       </c>
@@ -6725,7 +6734,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>34</v>
       </c>
@@ -6733,7 +6742,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
         <v>36</v>
       </c>
@@ -6741,7 +6750,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
         <v>39</v>
       </c>
@@ -6749,7 +6758,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
         <v>41</v>
       </c>
@@ -6757,7 +6766,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
         <v>44</v>
       </c>
@@ -6765,7 +6774,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
         <v>47</v>
       </c>
@@ -6773,7 +6782,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
         <v>49</v>
       </c>
@@ -6781,7 +6790,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
         <v>51</v>
       </c>
@@ -6789,7 +6798,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
         <v>54</v>
       </c>
@@ -6797,7 +6806,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
         <v>56</v>
       </c>
@@ -6805,7 +6814,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
         <v>60</v>
       </c>
@@ -6813,7 +6822,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
         <v>62</v>
       </c>
@@ -6821,7 +6830,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
         <v>64</v>
       </c>
@@ -6829,7 +6838,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
         <v>67</v>
       </c>
@@ -6837,7 +6846,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B25" t="s">
         <v>69</v>
       </c>
@@ -6845,7 +6854,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
         <v>72</v>
       </c>
@@ -6853,7 +6862,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B27" t="s">
         <v>74</v>
       </c>
@@ -6861,7 +6870,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B28" t="s">
         <v>77</v>
       </c>
@@ -6869,7 +6878,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B29" t="s">
         <v>79</v>
       </c>
@@ -6877,7 +6886,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="30" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
         <v>82</v>
       </c>
@@ -6885,7 +6894,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="31" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="31" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B31" t="s">
         <v>84</v>
       </c>
@@ -6893,7 +6902,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
         <v>86</v>
       </c>
@@ -6901,7 +6910,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B33" t="s">
         <v>89</v>
       </c>
@@ -6909,7 +6918,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
         <v>91</v>
       </c>
@@ -6917,7 +6926,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B35" t="s">
         <v>95</v>
       </c>
@@ -6925,7 +6934,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
         <v>98</v>
       </c>
@@ -6933,7 +6942,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
         <v>101</v>
       </c>
@@ -6941,7 +6950,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B38" t="s">
         <v>103</v>
       </c>
@@ -6949,7 +6958,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B39" t="s">
         <v>456</v>
       </c>
@@ -6957,7 +6966,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B40" t="s">
         <v>105</v>
       </c>
@@ -6965,7 +6974,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="41" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B41" t="s">
         <v>107</v>
       </c>
@@ -6973,7 +6982,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="42" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="42" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B42" t="s">
         <v>109</v>
       </c>
@@ -6981,7 +6990,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="43" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B43" t="s">
         <v>112</v>
       </c>
@@ -6989,7 +6998,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="44" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="44" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B44" t="s">
         <v>115</v>
       </c>
@@ -6997,7 +7006,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="45" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="45" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B45" t="s">
         <v>118</v>
       </c>
@@ -7005,7 +7014,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="46" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="46" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B46" t="s">
         <v>121</v>
       </c>
@@ -7013,7 +7022,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="47" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B47" t="s">
         <v>123</v>
       </c>
@@ -7021,7 +7030,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="48" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B48" t="s">
         <v>125</v>
       </c>
@@ -7029,7 +7038,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="49" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B49" t="s">
         <v>128</v>
       </c>
@@ -7037,7 +7046,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="50" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="50" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B50" t="s">
         <v>130</v>
       </c>
@@ -7045,7 +7054,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="51" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="51" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B51" t="s">
         <v>132</v>
       </c>
@@ -7053,7 +7062,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="52" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="52" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B52" t="s">
         <v>134</v>
       </c>
@@ -7061,7 +7070,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="53" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="53" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B53" t="s">
         <v>136</v>
       </c>
@@ -7069,7 +7078,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="54" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="54" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B54" t="s">
         <v>370</v>
       </c>
@@ -7077,7 +7086,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="55" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="55" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B55" t="s">
         <v>141</v>
       </c>
@@ -7085,7 +7094,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="56" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="56" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B56" t="s">
         <v>144</v>
       </c>
@@ -7093,7 +7102,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="57" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="57" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B57" t="s">
         <v>147</v>
       </c>
@@ -7101,7 +7110,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="58" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="58" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B58" t="s">
         <v>149</v>
       </c>
@@ -7109,7 +7118,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="59" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="59" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B59" t="s">
         <v>152</v>
       </c>
@@ -7117,7 +7126,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="60" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="60" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B60" t="s">
         <v>154</v>
       </c>
@@ -7125,7 +7134,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="61" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="61" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B61" t="s">
         <v>156</v>
       </c>
@@ -7133,7 +7142,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="62" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="62" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B62" t="s">
         <v>158</v>
       </c>
@@ -7141,7 +7150,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="63" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="63" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B63" t="s">
         <v>161</v>
       </c>
@@ -7149,7 +7158,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="64" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="64" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B64" t="s">
         <v>163</v>
       </c>
@@ -7157,7 +7166,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="65" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="65" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B65" t="s">
         <v>165</v>
       </c>
@@ -7165,7 +7174,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="66" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="66" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B66" t="s">
         <v>167</v>
       </c>
@@ -7173,7 +7182,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="67" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="67" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B67" t="s">
         <v>169</v>
       </c>
@@ -7181,7 +7190,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="68" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="68" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B68" t="s">
         <v>457</v>
       </c>
@@ -7189,7 +7198,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="69" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="69" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B69" t="s">
         <v>172</v>
       </c>
@@ -7197,7 +7206,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="70" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="70" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B70" t="s">
         <v>175</v>
       </c>
@@ -7205,7 +7214,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="71" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="71" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B71" t="s">
         <v>177</v>
       </c>
@@ -7213,7 +7222,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="72" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="72" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B72" t="s">
         <v>179</v>
       </c>
@@ -7221,7 +7230,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="73" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="73" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B73" t="s">
         <v>181</v>
       </c>
@@ -7229,7 +7238,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="74" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="74" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B74" t="s">
         <v>183</v>
       </c>
@@ -7237,7 +7246,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="75" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="75" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B75" t="s">
         <v>186</v>
       </c>
@@ -7245,7 +7254,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="76" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="76" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B76" t="s">
         <v>189</v>
       </c>
@@ -7253,7 +7262,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="77" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="77" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B77" t="s">
         <v>191</v>
       </c>
@@ -7261,7 +7270,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="78" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="78" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B78" t="s">
         <v>193</v>
       </c>
@@ -7269,7 +7278,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="79" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="79" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B79" t="s">
         <v>195</v>
       </c>
@@ -7277,7 +7286,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="80" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="80" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B80" t="s">
         <v>197</v>
       </c>
@@ -7292,4 +7301,10 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{95965d95-ecc0-4720-b759-1f33c42ed7da}" enabled="1" method="Standard" siteId="{a0f29d7e-28cd-4f54-8442-7885aee7c080}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
update .xlsx to use crystallizer for name
</commit_message>
<xml_diff>
--- a/docs/technical_reference/unit_models/zero_order_unit_models/WT3_unit_classification_for_doc.xlsx
+++ b/docs/technical_reference/unit_models/zero_order_unit_models/WT3_unit_classification_for_doc.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10517"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35874F6C-7701-DF4B-AA7A-C888519018C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{864AF8A0-179E-0449-9BD5-7605F6307A2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="515">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="516">
   <si>
     <t>Name</t>
   </si>
@@ -1577,6 +1577,9 @@
   </si>
   <si>
     <t>cost_crystallizer</t>
+  </si>
+  <si>
+    <t>crystallizer</t>
   </si>
 </sst>
 </file>
@@ -2895,7 +2898,7 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>28</v>
+        <v>515</v>
       </c>
       <c r="B28" t="s">
         <v>512</v>

</xml_diff>

<commit_message>
fix docx merge conflicts
</commit_message>
<xml_diff>
--- a/docs/technical_reference/unit_models/zero_order_unit_models/WT3_unit_classification_for_doc.xlsx
+++ b/docs/technical_reference/unit_models/zero_order_unit_models/WT3_unit_classification_for_doc.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10531"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{864AF8A0-179E-0449-9BD5-7605F6307A2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7C1B3F5-E496-E348-B5C9-5A5374BB4600}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10580" yWindow="2740" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -13,7 +13,7 @@
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$92</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="516">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1000" uniqueCount="515">
   <si>
     <t>Name</t>
   </si>
@@ -419,9 +419,6 @@
   </si>
   <si>
     <t>microfiltration_zo</t>
-  </si>
-  <si>
-    <t>microscreen filtration</t>
   </si>
   <si>
     <t>microscreen_filtration_zo</t>
@@ -1953,7 +1950,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J93"/>
+  <dimension ref="A1:J92"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="33.5" customWidth="1"/>
@@ -1975,7 +1972,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
@@ -1984,7 +1981,7 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="G1" t="s">
         <v>4</v>
@@ -2007,7 +2004,7 @@
         <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="D2" t="s">
         <v>10</v>
@@ -2042,7 +2039,7 @@
         <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="D3" t="s">
         <v>10</v>
@@ -2071,13 +2068,13 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="B4" t="s">
         <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="D4" t="s">
         <v>10</v>
@@ -2106,13 +2103,13 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>462</v>
+      </c>
+      <c r="B5" t="s">
         <v>463</v>
       </c>
-      <c r="B5" t="s">
-        <v>464</v>
-      </c>
       <c r="C5" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D5" t="s">
         <v>30</v>
@@ -2146,7 +2143,7 @@
         <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="D6" t="s">
         <v>30</v>
@@ -2161,7 +2158,7 @@
         <v>21</v>
       </c>
       <c r="H6" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="I6" t="str">
         <f t="shared" si="1"/>
@@ -2174,13 +2171,13 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="B7" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C7" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="D7" t="s">
         <v>30</v>
@@ -2195,7 +2192,7 @@
         <v>31</v>
       </c>
       <c r="H7" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="I7" t="str">
         <f t="shared" si="1"/>
@@ -2214,7 +2211,7 @@
         <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -2249,7 +2246,7 @@
         <v>23</v>
       </c>
       <c r="C9" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="D9" t="s">
         <v>10</v>
@@ -2284,7 +2281,7 @@
         <v>25</v>
       </c>
       <c r="C10" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D10" t="s">
         <v>10</v>
@@ -2313,13 +2310,13 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B11" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C11" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="D11" t="s">
         <v>10</v>
@@ -2354,7 +2351,7 @@
         <v>29</v>
       </c>
       <c r="C12" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="D12" t="s">
         <v>30</v>
@@ -2388,7 +2385,7 @@
         <v>34</v>
       </c>
       <c r="C13" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D13" t="s">
         <v>10</v>
@@ -2423,7 +2420,7 @@
         <v>36</v>
       </c>
       <c r="C14" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="D14" t="s">
         <v>30</v>
@@ -2457,7 +2454,7 @@
         <v>39</v>
       </c>
       <c r="C15" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="D15" t="s">
         <v>10</v>
@@ -2486,13 +2483,13 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>466</v>
+      </c>
+      <c r="B16" t="s">
         <v>467</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>468</v>
-      </c>
-      <c r="C16" t="s">
-        <v>469</v>
       </c>
       <c r="D16" t="s">
         <v>30</v>
@@ -2507,7 +2504,7 @@
         <v>12</v>
       </c>
       <c r="H16" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="I16" t="str">
         <f t="shared" si="1"/>
@@ -2526,7 +2523,7 @@
         <v>41</v>
       </c>
       <c r="C17" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D17" t="s">
         <v>30</v>
@@ -2560,7 +2557,7 @@
         <v>44</v>
       </c>
       <c r="C18" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="D18" t="s">
         <v>30</v>
@@ -2594,7 +2591,7 @@
         <v>47</v>
       </c>
       <c r="C19" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="D19" t="s">
         <v>10</v>
@@ -2623,13 +2620,13 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>470</v>
+      </c>
+      <c r="B20" t="s">
         <v>471</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>472</v>
-      </c>
-      <c r="C20" t="s">
-        <v>473</v>
       </c>
       <c r="D20" t="s">
         <v>10</v>
@@ -2663,7 +2660,7 @@
         <v>49</v>
       </c>
       <c r="C21" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="D21" t="s">
         <v>10</v>
@@ -2698,7 +2695,7 @@
         <v>51</v>
       </c>
       <c r="C22" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D22" t="s">
         <v>30</v>
@@ -2732,7 +2729,7 @@
         <v>54</v>
       </c>
       <c r="C23" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="D23" t="s">
         <v>30</v>
@@ -2747,7 +2744,7 @@
         <v>21</v>
       </c>
       <c r="H23" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="I23" t="str">
         <f t="shared" si="1"/>
@@ -2766,7 +2763,7 @@
         <v>56</v>
       </c>
       <c r="C24" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="D24" t="s">
         <v>30</v>
@@ -2781,7 +2778,7 @@
         <v>58</v>
       </c>
       <c r="H24" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="I24" t="str">
         <f t="shared" si="1"/>
@@ -2800,7 +2797,7 @@
         <v>60</v>
       </c>
       <c r="C25" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="D25" t="s">
         <v>10</v>
@@ -2835,7 +2832,7 @@
         <v>62</v>
       </c>
       <c r="C26" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="D26" t="s">
         <v>10</v>
@@ -2870,7 +2867,7 @@
         <v>64</v>
       </c>
       <c r="C27" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="D27" t="s">
         <v>30</v>
@@ -2898,13 +2895,13 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B28" t="s">
+        <v>511</v>
+      </c>
+      <c r="C28" t="s">
         <v>512</v>
-      </c>
-      <c r="C28" t="s">
-        <v>513</v>
       </c>
       <c r="D28" t="s">
         <v>30</v>
@@ -2919,7 +2916,7 @@
         <v>31</v>
       </c>
       <c r="H28" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="I28" t="str">
         <f t="shared" ref="I28" si="3">IF(E28="SIDO","single-input, double-output",IF(E28="SISO","single-input, single-output",IF(E28="PT","pass-through",IF(E28="DISO","double-input, single-output",IF(E28="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
@@ -2938,7 +2935,7 @@
         <v>67</v>
       </c>
       <c r="C29" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="D29" t="s">
         <v>10</v>
@@ -2973,7 +2970,7 @@
         <v>69</v>
       </c>
       <c r="C30" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="D30" t="s">
         <v>30</v>
@@ -3007,7 +3004,7 @@
         <v>72</v>
       </c>
       <c r="C31" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D31" t="s">
         <v>10</v>
@@ -3042,7 +3039,7 @@
         <v>74</v>
       </c>
       <c r="C32" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="D32" t="s">
         <v>57</v>
@@ -3076,7 +3073,7 @@
         <v>77</v>
       </c>
       <c r="C33" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="D33" t="s">
         <v>10</v>
@@ -3111,7 +3108,7 @@
         <v>79</v>
       </c>
       <c r="C34" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="D34" t="s">
         <v>30</v>
@@ -3139,13 +3136,13 @@
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
+        <v>507</v>
+      </c>
+      <c r="B35" t="s">
         <v>508</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
         <v>509</v>
-      </c>
-      <c r="C35" t="s">
-        <v>510</v>
       </c>
       <c r="D35" t="s">
         <v>30</v>
@@ -3160,7 +3157,7 @@
         <v>31</v>
       </c>
       <c r="H35" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="I35" t="str">
         <f t="shared" si="1"/>
@@ -3179,7 +3176,7 @@
         <v>82</v>
       </c>
       <c r="C36" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="D36" t="s">
         <v>30</v>
@@ -3213,7 +3210,7 @@
         <v>84</v>
       </c>
       <c r="C37" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="D37" t="s">
         <v>10</v>
@@ -3248,7 +3245,7 @@
         <v>86</v>
       </c>
       <c r="C38" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="D38" t="s">
         <v>30</v>
@@ -3282,7 +3279,7 @@
         <v>89</v>
       </c>
       <c r="C39" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D39" t="s">
         <v>10</v>
@@ -3317,7 +3314,7 @@
         <v>91</v>
       </c>
       <c r="C40" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D40" t="s">
         <v>92</v>
@@ -3350,7 +3347,7 @@
         <v>95</v>
       </c>
       <c r="C41" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="D41" t="s">
         <v>30</v>
@@ -3384,7 +3381,7 @@
         <v>98</v>
       </c>
       <c r="C42" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D42" t="s">
         <v>30</v>
@@ -3418,7 +3415,7 @@
         <v>101</v>
       </c>
       <c r="C43" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="D43" t="s">
         <v>30</v>
@@ -3433,7 +3430,7 @@
         <v>31</v>
       </c>
       <c r="H43" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="I43" t="str">
         <f t="shared" si="5"/>
@@ -3452,7 +3449,7 @@
         <v>103</v>
       </c>
       <c r="C44" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="D44" t="s">
         <v>30</v>
@@ -3480,13 +3477,13 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
+        <v>474</v>
+      </c>
+      <c r="B45" t="s">
+        <v>473</v>
+      </c>
+      <c r="C45" t="s">
         <v>475</v>
-      </c>
-      <c r="B45" t="s">
-        <v>474</v>
-      </c>
-      <c r="C45" t="s">
-        <v>476</v>
       </c>
       <c r="D45" t="s">
         <v>10</v>
@@ -3501,7 +3498,7 @@
         <v>12</v>
       </c>
       <c r="H45" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="I45" t="str">
         <f t="shared" si="5"/>
@@ -3514,13 +3511,13 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B46" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="C46" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="D46" t="s">
         <v>30</v>
@@ -3535,7 +3532,7 @@
         <v>31</v>
       </c>
       <c r="H46" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="I46" t="str">
         <f t="shared" si="5"/>
@@ -3554,7 +3551,7 @@
         <v>105</v>
       </c>
       <c r="C47" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="D47" t="s">
         <v>10</v>
@@ -3573,11 +3570,11 @@
         <v>cost_power_law_flow</v>
       </c>
       <c r="I47" t="str">
-        <f t="shared" ref="I47:I93" si="7">IF(E47="SIDO","single-input, double-output",IF(E47="SISO","single-input, single-output",IF(E47="PT","pass-through",IF(E47="DISO","double-input, single-output",IF(E47="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
+        <f t="shared" ref="I47:I92" si="7">IF(E47="SIDO","single-input, double-output",IF(E47="SISO","single-input, single-output",IF(E47="PT","pass-through",IF(E47="DISO","double-input, single-output",IF(E47="SIDO reactive","reactive single-inlet, double-outlet","")))))</f>
         <v>pass-through</v>
       </c>
       <c r="J47" t="str">
-        <f t="shared" ref="J47:J93" si="8">IF(E47="SIDO","sido_methods",IF(E47="SISO","siso_methods",IF(E47="PT","pt_methods",IF(E47="DISO","diso_methods",IF(E47="SIDO reactive","sidor_methods","")))))</f>
+        <f t="shared" ref="J47:J92" si="8">IF(E47="SIDO","sido_methods",IF(E47="SISO","siso_methods",IF(E47="PT","pt_methods",IF(E47="DISO","diso_methods",IF(E47="SIDO reactive","sidor_methods","")))))</f>
         <v>pt_methods</v>
       </c>
     </row>
@@ -3589,7 +3586,7 @@
         <v>107</v>
       </c>
       <c r="C48" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="D48" t="s">
         <v>10</v>
@@ -3624,7 +3621,7 @@
         <v>109</v>
       </c>
       <c r="C49" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="D49" t="s">
         <v>30</v>
@@ -3658,7 +3655,7 @@
         <v>112</v>
       </c>
       <c r="C50" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="D50" t="s">
         <v>30</v>
@@ -3692,7 +3689,7 @@
         <v>115</v>
       </c>
       <c r="C51" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D51" t="s">
         <v>10</v>
@@ -3726,7 +3723,7 @@
         <v>118</v>
       </c>
       <c r="C52" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="D52" t="s">
         <v>30</v>
@@ -3754,13 +3751,13 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
+        <v>479</v>
+      </c>
+      <c r="B53" t="s">
         <v>480</v>
       </c>
-      <c r="B53" t="s">
+      <c r="C53" t="s">
         <v>481</v>
-      </c>
-      <c r="C53" t="s">
-        <v>482</v>
       </c>
       <c r="D53" t="s">
         <v>30</v>
@@ -3775,7 +3772,7 @@
         <v>12</v>
       </c>
       <c r="H53" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="I53" t="str">
         <f t="shared" si="7"/>
@@ -3794,7 +3791,7 @@
         <v>121</v>
       </c>
       <c r="C54" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="D54" t="s">
         <v>10</v>
@@ -3829,7 +3826,7 @@
         <v>123</v>
       </c>
       <c r="C55" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="D55" t="s">
         <v>10</v>
@@ -3858,13 +3855,13 @@
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
+        <v>483</v>
+      </c>
+      <c r="B56" t="s">
         <v>484</v>
       </c>
-      <c r="B56" t="s">
+      <c r="C56" t="s">
         <v>485</v>
-      </c>
-      <c r="C56" t="s">
-        <v>486</v>
       </c>
       <c r="D56" t="s">
         <v>30</v>
@@ -3879,7 +3876,7 @@
         <v>12</v>
       </c>
       <c r="H56" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="I56" t="str">
         <f t="shared" si="7"/>
@@ -3898,7 +3895,7 @@
         <v>125</v>
       </c>
       <c r="C57" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="D57" t="s">
         <v>30</v>
@@ -3926,13 +3923,13 @@
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
+        <v>487</v>
+      </c>
+      <c r="B58" t="s">
         <v>488</v>
       </c>
-      <c r="B58" t="s">
+      <c r="C58" t="s">
         <v>489</v>
-      </c>
-      <c r="C58" t="s">
-        <v>490</v>
       </c>
       <c r="D58" t="s">
         <v>30</v>
@@ -3947,7 +3944,7 @@
         <v>12</v>
       </c>
       <c r="H58" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="I58" t="str">
         <f t="shared" si="7"/>
@@ -3966,7 +3963,7 @@
         <v>128</v>
       </c>
       <c r="C59" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="D59" t="s">
         <v>10</v>
@@ -3995,48 +3992,47 @@
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B60" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C60" t="s">
-        <v>404</v>
+        <v>423</v>
       </c>
       <c r="D60" t="s">
         <v>10</v>
       </c>
       <c r="E60" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F60" t="b">
         <v>1</v>
       </c>
       <c r="G60" t="s">
-        <v>12</v>
-      </c>
-      <c r="H60" t="str">
-        <f>IF(D60="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+        <v>21</v>
+      </c>
+      <c r="H60" t="s">
+        <v>65</v>
       </c>
       <c r="I60" t="str">
         <f t="shared" si="7"/>
-        <v>single-input, double-output</v>
+        <v>pass-through</v>
       </c>
       <c r="J60" t="str">
         <f t="shared" si="8"/>
-        <v>sido_methods</v>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B61" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C61" t="s">
-        <v>424</v>
+        <v>404</v>
       </c>
       <c r="D61" t="s">
         <v>10</v>
@@ -4048,10 +4044,11 @@
         <v>1</v>
       </c>
       <c r="G61" t="s">
-        <v>21</v>
-      </c>
-      <c r="H61" t="s">
-        <v>65</v>
+        <v>12</v>
+      </c>
+      <c r="H61" t="str">
+        <f>IF(D61="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I61" t="str">
         <f t="shared" si="7"/>
@@ -4064,54 +4061,53 @@
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B62" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C62" t="s">
         <v>405</v>
       </c>
       <c r="D62" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E62" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F62" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G62" t="s">
-        <v>12</v>
-      </c>
-      <c r="H62" t="str">
-        <f>IF(D62="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+        <v>31</v>
+      </c>
+      <c r="H62" t="s">
+        <v>136</v>
       </c>
       <c r="I62" t="str">
         <f t="shared" si="7"/>
-        <v>pass-through</v>
+        <v>single-input, double-output</v>
       </c>
       <c r="J62" t="str">
         <f t="shared" si="8"/>
-        <v>pt_methods</v>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B63" t="s">
-        <v>136</v>
+        <v>369</v>
       </c>
       <c r="C63" t="s">
-        <v>406</v>
+        <v>425</v>
       </c>
       <c r="D63" t="s">
         <v>30</v>
       </c>
       <c r="E63" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F63" t="b">
         <v>0</v>
@@ -4120,26 +4116,26 @@
         <v>31</v>
       </c>
       <c r="H63" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I63" t="str">
         <f t="shared" si="7"/>
-        <v>single-input, double-output</v>
+        <v>single-input, single-output</v>
       </c>
       <c r="J63" t="str">
         <f t="shared" si="8"/>
-        <v>sido_methods</v>
+        <v>siso_methods</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B64" t="s">
-        <v>370</v>
+        <v>140</v>
       </c>
       <c r="C64" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D64" t="s">
         <v>30</v>
@@ -4154,7 +4150,7 @@
         <v>31</v>
       </c>
       <c r="H64" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="I64" t="str">
         <f t="shared" si="7"/>
@@ -4167,96 +4163,97 @@
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>140</v>
+        <v>491</v>
       </c>
       <c r="B65" t="s">
-        <v>141</v>
+        <v>492</v>
       </c>
       <c r="C65" t="s">
-        <v>425</v>
+        <v>493</v>
       </c>
       <c r="D65" t="s">
         <v>30</v>
       </c>
       <c r="E65" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="F65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G65" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="H65" t="s">
-        <v>142</v>
+        <v>494</v>
       </c>
       <c r="I65" t="str">
         <f t="shared" si="7"/>
-        <v>single-input, single-output</v>
+        <v>reactive single-inlet, double-outlet</v>
       </c>
       <c r="J65" t="str">
         <f t="shared" si="8"/>
-        <v>siso_methods</v>
+        <v>sidor_methods</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>492</v>
+        <v>142</v>
       </c>
       <c r="B66" t="s">
-        <v>493</v>
+        <v>143</v>
       </c>
       <c r="C66" t="s">
-        <v>494</v>
+        <v>443</v>
       </c>
       <c r="D66" t="s">
         <v>30</v>
       </c>
       <c r="E66" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F66" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G66" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="H66" t="s">
-        <v>495</v>
+        <v>144</v>
       </c>
       <c r="I66" t="str">
         <f t="shared" si="7"/>
-        <v>reactive single-inlet, double-outlet</v>
+        <v>single-input, double-output</v>
       </c>
       <c r="J66" t="str">
         <f t="shared" si="8"/>
-        <v>sidor_methods</v>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B67" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C67" t="s">
-        <v>444</v>
+        <v>407</v>
       </c>
       <c r="D67" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E67" t="s">
         <v>11</v>
       </c>
       <c r="F67" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G67" t="s">
-        <v>31</v>
-      </c>
-      <c r="H67" t="s">
-        <v>145</v>
+        <v>12</v>
+      </c>
+      <c r="H67" t="str">
+        <f>IF(D67="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I67" t="str">
         <f t="shared" si="7"/>
@@ -4269,63 +4266,63 @@
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B68" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C68" t="s">
-        <v>408</v>
+        <v>398</v>
       </c>
       <c r="D68" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E68" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F68" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G68" t="s">
-        <v>12</v>
-      </c>
-      <c r="H68" t="str">
-        <f>IF(D68="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+        <v>31</v>
+      </c>
+      <c r="H68" t="s">
+        <v>149</v>
       </c>
       <c r="I68" t="str">
         <f t="shared" si="7"/>
-        <v>single-input, double-output</v>
+        <v>pass-through</v>
       </c>
       <c r="J68" t="str">
         <f t="shared" si="8"/>
-        <v>sido_methods</v>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B69" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C69" t="s">
-        <v>399</v>
+        <v>408</v>
       </c>
       <c r="D69" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E69" t="s">
         <v>27</v>
       </c>
       <c r="F69" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G69" t="s">
-        <v>31</v>
-      </c>
-      <c r="H69" t="s">
-        <v>150</v>
+        <v>12</v>
+      </c>
+      <c r="H69" t="str">
+        <f>IF(D69="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I69" t="str">
         <f t="shared" si="7"/>
@@ -4338,10 +4335,10 @@
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B70" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C70" t="s">
         <v>409</v>
@@ -4350,7 +4347,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F70" t="b">
         <v>1</v>
@@ -4364,25 +4361,25 @@
       </c>
       <c r="I70" t="str">
         <f t="shared" si="7"/>
-        <v>pass-through</v>
+        <v>single-input, double-output</v>
       </c>
       <c r="J70" t="str">
         <f t="shared" si="8"/>
-        <v>pt_methods</v>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B71" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C71" t="s">
-        <v>410</v>
+        <v>447</v>
       </c>
       <c r="D71" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="E71" t="s">
         <v>11</v>
@@ -4393,9 +4390,8 @@
       <c r="G71" t="s">
         <v>12</v>
       </c>
-      <c r="H71" t="str">
-        <f>IF(D71="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H71" t="s">
+        <v>65</v>
       </c>
       <c r="I71" t="str">
         <f t="shared" si="7"/>
@@ -4408,16 +4404,16 @@
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B72" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C72" t="s">
-        <v>448</v>
+        <v>410</v>
       </c>
       <c r="D72" t="s">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="E72" t="s">
         <v>11</v>
@@ -4429,7 +4425,7 @@
         <v>12</v>
       </c>
       <c r="H72" t="s">
-        <v>65</v>
+        <v>158</v>
       </c>
       <c r="I72" t="str">
         <f t="shared" si="7"/>
@@ -4442,16 +4438,16 @@
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B73" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C73" t="s">
         <v>411</v>
       </c>
       <c r="D73" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E73" t="s">
         <v>11</v>
@@ -4462,8 +4458,9 @@
       <c r="G73" t="s">
         <v>12</v>
       </c>
-      <c r="H73" t="s">
-        <v>159</v>
+      <c r="H73" t="str">
+        <f>IF(D73="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I73" t="str">
         <f t="shared" si="7"/>
@@ -4476,13 +4473,13 @@
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B74" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C74" t="s">
-        <v>412</v>
+        <v>435</v>
       </c>
       <c r="D74" t="s">
         <v>10</v>
@@ -4511,19 +4508,19 @@
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B75" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C75" t="s">
-        <v>436</v>
+        <v>412</v>
       </c>
       <c r="D75" t="s">
         <v>10</v>
       </c>
       <c r="E75" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F75" t="b">
         <v>1</v>
@@ -4537,22 +4534,22 @@
       </c>
       <c r="I75" t="str">
         <f t="shared" si="7"/>
-        <v>single-input, double-output</v>
+        <v>pass-through</v>
       </c>
       <c r="J75" t="str">
         <f t="shared" si="8"/>
-        <v>sido_methods</v>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B76" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C76" t="s">
-        <v>413</v>
+        <v>433</v>
       </c>
       <c r="D76" t="s">
         <v>10</v>
@@ -4581,16 +4578,16 @@
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B77" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C77" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="D77" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E77" t="s">
         <v>27</v>
@@ -4601,9 +4598,8 @@
       <c r="G77" t="s">
         <v>12</v>
       </c>
-      <c r="H77" t="str">
-        <f>IF(D77="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H77" t="s">
+        <v>169</v>
       </c>
       <c r="I77" t="str">
         <f t="shared" si="7"/>
@@ -4616,16 +4612,16 @@
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>168</v>
+        <v>495</v>
       </c>
       <c r="B78" t="s">
-        <v>169</v>
+        <v>496</v>
       </c>
       <c r="C78" t="s">
-        <v>431</v>
+        <v>497</v>
       </c>
       <c r="D78" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E78" t="s">
         <v>27</v>
@@ -4637,7 +4633,7 @@
         <v>12</v>
       </c>
       <c r="H78" t="s">
-        <v>170</v>
+        <v>498</v>
       </c>
       <c r="I78" t="str">
         <f t="shared" si="7"/>
@@ -4650,19 +4646,19 @@
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="B79" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="C79" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="D79" t="s">
         <v>10</v>
       </c>
       <c r="E79" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F79" t="b">
         <v>1</v>
@@ -4671,41 +4667,41 @@
         <v>12</v>
       </c>
       <c r="H79" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="I79" t="str">
         <f t="shared" si="7"/>
-        <v>pass-through</v>
+        <v>single-input, double-output</v>
       </c>
       <c r="J79" t="str">
         <f t="shared" si="8"/>
-        <v>pt_methods</v>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="B80" t="s">
-        <v>501</v>
+        <v>456</v>
       </c>
       <c r="C80" t="s">
-        <v>502</v>
+        <v>452</v>
       </c>
       <c r="D80" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E80" t="s">
         <v>11</v>
       </c>
       <c r="F80" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G80" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="H80" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="I80" t="str">
         <f t="shared" si="7"/>
@@ -4718,50 +4714,50 @@
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>504</v>
+        <v>170</v>
       </c>
       <c r="B81" t="s">
-        <v>457</v>
+        <v>171</v>
       </c>
       <c r="C81" t="s">
-        <v>453</v>
+        <v>442</v>
       </c>
       <c r="D81" t="s">
         <v>30</v>
       </c>
       <c r="E81" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F81" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G81" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="H81" t="s">
-        <v>505</v>
+        <v>172</v>
       </c>
       <c r="I81" t="str">
         <f t="shared" si="7"/>
-        <v>single-input, double-output</v>
+        <v>pass-through</v>
       </c>
       <c r="J81" t="str">
         <f t="shared" si="8"/>
-        <v>sido_methods</v>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B82" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C82" t="s">
-        <v>443</v>
+        <v>431</v>
       </c>
       <c r="D82" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E82" t="s">
         <v>27</v>
@@ -4772,8 +4768,9 @@
       <c r="G82" t="s">
         <v>21</v>
       </c>
-      <c r="H82" t="s">
-        <v>173</v>
+      <c r="H82" t="str">
+        <f>IF(D82="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I82" t="str">
         <f t="shared" si="7"/>
@@ -4786,13 +4783,13 @@
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B83" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C83" t="s">
-        <v>432</v>
+        <v>413</v>
       </c>
       <c r="D83" t="s">
         <v>10</v>
@@ -4804,7 +4801,7 @@
         <v>1</v>
       </c>
       <c r="G83" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="H83" t="str">
         <f>IF(D83="basic","cost_power_law_flow")</f>
@@ -4821,10 +4818,10 @@
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B84" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C84" t="s">
         <v>414</v>
@@ -4833,7 +4830,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F84" t="b">
         <v>1</v>
@@ -4847,22 +4844,22 @@
       </c>
       <c r="I84" t="str">
         <f t="shared" si="7"/>
-        <v>pass-through</v>
+        <v>single-input, double-output</v>
       </c>
       <c r="J84" t="str">
         <f t="shared" si="8"/>
-        <v>pt_methods</v>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B85" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C85" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D85" t="s">
         <v>10</v>
@@ -4891,19 +4888,19 @@
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B86" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C86" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D86" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E86" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="F86" t="b">
         <v>1</v>
@@ -4911,28 +4908,27 @@
       <c r="G86" t="s">
         <v>12</v>
       </c>
-      <c r="H86" t="str">
-        <f>IF(D86="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+      <c r="H86" t="s">
+        <v>183</v>
       </c>
       <c r="I86" t="str">
         <f t="shared" si="7"/>
-        <v>single-input, double-output</v>
+        <v>single-input, single-output</v>
       </c>
       <c r="J86" t="str">
         <f t="shared" si="8"/>
-        <v>sido_methods</v>
+        <v>siso_methods</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B87" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C87" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="D87" t="s">
         <v>30</v>
@@ -4947,7 +4943,7 @@
         <v>12</v>
       </c>
       <c r="H87" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="I87" t="str">
         <f t="shared" si="7"/>
@@ -4960,19 +4956,19 @@
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B88" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C88" t="s">
-        <v>418</v>
+        <v>453</v>
       </c>
       <c r="D88" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="E88" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F88" t="b">
         <v>1</v>
@@ -4981,29 +4977,29 @@
         <v>12</v>
       </c>
       <c r="H88" t="s">
-        <v>187</v>
+        <v>460</v>
       </c>
       <c r="I88" t="str">
         <f t="shared" si="7"/>
-        <v>single-input, single-output</v>
+        <v>single-input, double-output</v>
       </c>
       <c r="J88" t="str">
         <f t="shared" si="8"/>
-        <v>siso_methods</v>
+        <v>sido_methods</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B89" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C89" t="s">
-        <v>454</v>
+        <v>420</v>
       </c>
       <c r="D89" t="s">
-        <v>57</v>
+        <v>10</v>
       </c>
       <c r="E89" t="s">
         <v>11</v>
@@ -5014,8 +5010,9 @@
       <c r="G89" t="s">
         <v>12</v>
       </c>
-      <c r="H89" t="s">
-        <v>461</v>
+      <c r="H89" t="str">
+        <f>IF(D89="basic","cost_power_law_flow")</f>
+        <v>cost_power_law_flow</v>
       </c>
       <c r="I89" t="str">
         <f t="shared" si="7"/>
@@ -5028,13 +5025,13 @@
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B90" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C90" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D90" t="s">
         <v>10</v>
@@ -5063,45 +5060,44 @@
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B91" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C91" t="s">
-        <v>420</v>
+        <v>438</v>
       </c>
       <c r="D91" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E91" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F91" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G91" t="s">
-        <v>12</v>
-      </c>
-      <c r="H91" t="str">
-        <f>IF(D91="basic","cost_power_law_flow")</f>
-        <v>cost_power_law_flow</v>
+        <v>31</v>
+      </c>
+      <c r="H91" t="s">
+        <v>65</v>
       </c>
       <c r="I91" t="str">
         <f t="shared" si="7"/>
-        <v>single-input, double-output</v>
+        <v>pass-through</v>
       </c>
       <c r="J91" t="str">
         <f t="shared" si="8"/>
-        <v>sido_methods</v>
+        <v>pt_methods</v>
       </c>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B92" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C92" t="s">
         <v>439</v>
@@ -5113,13 +5109,13 @@
         <v>27</v>
       </c>
       <c r="F92" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G92" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="H92" t="s">
-        <v>65</v>
+        <v>197</v>
       </c>
       <c r="I92" t="str">
         <f t="shared" si="7"/>
@@ -5130,43 +5126,9 @@
         <v>pt_methods</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
-        <v>196</v>
-      </c>
-      <c r="B93" t="s">
-        <v>197</v>
-      </c>
-      <c r="C93" t="s">
-        <v>440</v>
-      </c>
-      <c r="D93" t="s">
-        <v>30</v>
-      </c>
-      <c r="E93" t="s">
-        <v>27</v>
-      </c>
-      <c r="F93" t="b">
-        <v>1</v>
-      </c>
-      <c r="G93" t="s">
-        <v>21</v>
-      </c>
-      <c r="H93" t="s">
-        <v>198</v>
-      </c>
-      <c r="I93" t="str">
-        <f t="shared" si="7"/>
-        <v>pass-through</v>
-      </c>
-      <c r="J93" t="str">
-        <f t="shared" si="8"/>
-        <v>pt_methods</v>
-      </c>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J93">
-    <sortCondition ref="B2:B93"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J92">
+    <sortCondition ref="B2:B92"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -5185,17 +5147,17 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B1" t="str">
         <f>CONCATENATE(A1,"_zo")</f>
         <v>aeration_basin_zo</v>
       </c>
       <c r="C1" t="s">
+        <v>199</v>
+      </c>
+      <c r="D1" t="s">
         <v>200</v>
-      </c>
-      <c r="D1" t="s">
-        <v>201</v>
       </c>
       <c r="G1" t="str">
         <f>CONCATENATE(C1," ",D1)</f>
@@ -5204,17 +5166,17 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B65" si="0">CONCATENATE(A2,"_zo")</f>
         <v>air_flotation_zo</v>
       </c>
       <c r="C2" t="s">
+        <v>202</v>
+      </c>
+      <c r="D2" t="s">
         <v>203</v>
-      </c>
-      <c r="D2" t="s">
-        <v>204</v>
       </c>
       <c r="G2" t="str">
         <f t="shared" ref="G2:G65" si="1">CONCATENATE(C2," ",D2)</f>
@@ -5223,20 +5185,20 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
         <v>anaerobic_digestion_oxidation_zo</v>
       </c>
       <c r="C3" t="s">
+        <v>205</v>
+      </c>
+      <c r="D3" t="s">
         <v>206</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>207</v>
-      </c>
-      <c r="E3" t="s">
-        <v>208</v>
       </c>
       <c r="G3" t="str">
         <f t="shared" si="1"/>
@@ -5245,20 +5207,20 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
         <v>anaerobic_mbr_mec_zo</v>
       </c>
       <c r="C4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D4" t="s">
+        <v>209</v>
+      </c>
+      <c r="E4" t="s">
         <v>210</v>
-      </c>
-      <c r="E4" t="s">
-        <v>211</v>
       </c>
       <c r="G4" t="str">
         <f>CONCATENATE(C4," ",D4," ",E4)</f>
@@ -5267,20 +5229,20 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
         <v>backwash_solids_handling_zo</v>
       </c>
       <c r="C5" t="s">
+        <v>212</v>
+      </c>
+      <c r="D5" t="s">
         <v>213</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>214</v>
-      </c>
-      <c r="E5" t="s">
-        <v>215</v>
       </c>
       <c r="G5" t="str">
         <f t="shared" ref="G5:G6" si="2">CONCATENATE(C5," ",D5," ",E5)</f>
@@ -5289,20 +5251,20 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
         <v>bio_active_filtration_zo</v>
       </c>
       <c r="C6" t="s">
+        <v>216</v>
+      </c>
+      <c r="D6" t="s">
         <v>217</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>218</v>
-      </c>
-      <c r="E6" t="s">
-        <v>219</v>
       </c>
       <c r="G6" t="str">
         <f t="shared" si="2"/>
@@ -5311,14 +5273,14 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
         <v>bioreactor_zo</v>
       </c>
       <c r="C7" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G7" t="str">
         <f t="shared" si="1"/>
@@ -5327,17 +5289,17 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
         <v>blending_resevoir_zo</v>
       </c>
       <c r="C8" t="s">
+        <v>221</v>
+      </c>
+      <c r="D8" t="s">
         <v>222</v>
-      </c>
-      <c r="D8" t="s">
-        <v>223</v>
       </c>
       <c r="G8" t="str">
         <f t="shared" si="1"/>
@@ -5346,17 +5308,17 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
         <v>brine_concentrator_zo</v>
       </c>
       <c r="C9" t="s">
+        <v>224</v>
+      </c>
+      <c r="D9" t="s">
         <v>225</v>
-      </c>
-      <c r="D9" t="s">
-        <v>226</v>
       </c>
       <c r="G9" t="str">
         <f t="shared" si="1"/>
@@ -5365,17 +5327,17 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
         <v>buffer_tank_zo</v>
       </c>
       <c r="C10" t="s">
+        <v>227</v>
+      </c>
+      <c r="D10" t="s">
         <v>228</v>
-      </c>
-      <c r="D10" t="s">
-        <v>229</v>
       </c>
       <c r="G10" t="str">
         <f t="shared" si="1"/>
@@ -5384,14 +5346,14 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
         <v>CANDOP_zo</v>
       </c>
       <c r="C11" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="G11" t="str">
         <f t="shared" si="1"/>
@@ -5400,17 +5362,17 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>cartridge_filtration_zo</v>
       </c>
       <c r="C12" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D12" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G12" t="str">
         <f t="shared" si="1"/>
@@ -5419,17 +5381,17 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v>chemical_addition_zo</v>
       </c>
       <c r="C13" t="s">
+        <v>233</v>
+      </c>
+      <c r="D13" t="s">
         <v>234</v>
-      </c>
-      <c r="D13" t="s">
-        <v>235</v>
       </c>
       <c r="G13" t="str">
         <f t="shared" si="1"/>
@@ -5438,14 +5400,14 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
         <v>chlorination_zo</v>
       </c>
       <c r="C14" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="G14" t="str">
         <f t="shared" si="1"/>
@@ -5454,14 +5416,14 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
         <v>clarifier_zo</v>
       </c>
       <c r="C15" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G15" t="str">
         <f t="shared" si="1"/>
@@ -5470,17 +5432,17 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
         <v>co2_addition_zo</v>
       </c>
       <c r="C16" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D16" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="G16" t="str">
         <f t="shared" si="1"/>
@@ -5489,20 +5451,20 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="0"/>
         <v>coag_and_floc_zo</v>
       </c>
       <c r="C17" t="s">
+        <v>240</v>
+      </c>
+      <c r="D17" t="s">
         <v>241</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>242</v>
-      </c>
-      <c r="E17" t="s">
-        <v>243</v>
       </c>
       <c r="G17" t="str">
         <f>CONCATENATE(C17," ",D17," ",E17)</f>
@@ -5511,14 +5473,14 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B18" t="str">
         <f t="shared" si="0"/>
         <v>cofermentation_zo</v>
       </c>
       <c r="C18" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="G18" t="str">
         <f t="shared" ref="G18:G19" si="3">CONCATENATE(C18," ",D18," ",E18)</f>
@@ -5527,17 +5489,17 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="0"/>
         <v>constructed_wetlands_zo</v>
       </c>
       <c r="C19" t="s">
+        <v>245</v>
+      </c>
+      <c r="D19" t="s">
         <v>246</v>
-      </c>
-      <c r="D19" t="s">
-        <v>247</v>
       </c>
       <c r="G19" t="str">
         <f t="shared" si="3"/>
@@ -5546,20 +5508,20 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B20" t="str">
         <f t="shared" si="0"/>
         <v>conventional_activated_sludge_zo</v>
       </c>
       <c r="C20" t="s">
+        <v>248</v>
+      </c>
+      <c r="D20" t="s">
         <v>249</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>250</v>
-      </c>
-      <c r="E20" t="s">
-        <v>251</v>
       </c>
       <c r="G20" t="str">
         <f>CONCATENATE(C20," ",D20," ",E20)</f>
@@ -5568,17 +5530,17 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B21" t="str">
         <f t="shared" si="0"/>
         <v>cooling_supply_zo</v>
       </c>
       <c r="C21" t="s">
+        <v>252</v>
+      </c>
+      <c r="D21" t="s">
         <v>253</v>
-      </c>
-      <c r="D21" t="s">
-        <v>254</v>
       </c>
       <c r="G21" t="str">
         <f t="shared" ref="G21:G22" si="4">CONCATENATE(C21," ",D21," ",E21)</f>
@@ -5587,17 +5549,17 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="0"/>
         <v>cooling_tower_zo</v>
       </c>
       <c r="C22" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D22" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G22" t="str">
         <f t="shared" si="4"/>
@@ -5606,14 +5568,14 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B23" t="str">
         <f t="shared" si="0"/>
         <v>decarbonator_zo</v>
       </c>
       <c r="C23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G23" t="str">
         <f t="shared" si="1"/>
@@ -5622,20 +5584,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B24" t="str">
         <f t="shared" si="0"/>
         <v>deep_well_injection_zo</v>
       </c>
       <c r="C24" t="s">
+        <v>258</v>
+      </c>
+      <c r="D24" t="s">
         <v>259</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>260</v>
-      </c>
-      <c r="E24" t="s">
-        <v>261</v>
       </c>
       <c r="G24" t="str">
         <f>CONCATENATE(C24," ",D24," ",E24)</f>
@@ -5644,20 +5606,20 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B25" t="str">
         <f t="shared" si="0"/>
         <v>dissolved_air_flotation_zo</v>
       </c>
       <c r="C25" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D25" t="s">
+        <v>202</v>
+      </c>
+      <c r="E25" t="s">
         <v>203</v>
-      </c>
-      <c r="E25" t="s">
-        <v>204</v>
       </c>
       <c r="G25" t="str">
         <f t="shared" ref="G25" si="5">CONCATENATE(C25," ",D25," ",E25)</f>
@@ -5666,14 +5628,14 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B26" t="str">
         <f t="shared" si="0"/>
         <v>dmbr_zo</v>
       </c>
       <c r="C26" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="G26" t="str">
         <f>CONCATENATE(C26," ",D26)</f>
@@ -5682,20 +5644,20 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B27" t="str">
         <f t="shared" si="0"/>
         <v>dual_media_filtration_zo</v>
       </c>
       <c r="C27" t="s">
+        <v>265</v>
+      </c>
+      <c r="D27" t="s">
         <v>266</v>
       </c>
-      <c r="D27" t="s">
-        <v>267</v>
-      </c>
       <c r="E27" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G27" t="str">
         <f>CONCATENATE(C27," ",D27," ",E27)</f>
@@ -5704,20 +5666,20 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="0"/>
         <v>electrochemical_nutrient_removal_zo</v>
       </c>
       <c r="C28" t="s">
+        <v>268</v>
+      </c>
+      <c r="D28" t="s">
         <v>269</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>270</v>
-      </c>
-      <c r="E28" t="s">
-        <v>271</v>
       </c>
       <c r="G28" t="str">
         <f>CONCATENATE(C28," ",D28," ",E28)</f>
@@ -5726,17 +5688,17 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="0"/>
         <v>electrodialysis_reversal_zo</v>
       </c>
       <c r="C29" t="s">
+        <v>272</v>
+      </c>
+      <c r="D29" t="s">
         <v>273</v>
-      </c>
-      <c r="D29" t="s">
-        <v>274</v>
       </c>
       <c r="G29" t="str">
         <f t="shared" si="1"/>
@@ -5745,7 +5707,7 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="0"/>
@@ -5755,7 +5717,7 @@
         <v>4</v>
       </c>
       <c r="D30" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="G30" t="str">
         <f t="shared" si="1"/>
@@ -5764,17 +5726,17 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="0"/>
         <v>evaporation_pond_zo</v>
       </c>
       <c r="C31" t="s">
+        <v>277</v>
+      </c>
+      <c r="D31" t="s">
         <v>278</v>
-      </c>
-      <c r="D31" t="s">
-        <v>279</v>
       </c>
       <c r="G31" t="str">
         <f t="shared" si="1"/>
@@ -5783,20 +5745,20 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B32" t="str">
         <f t="shared" si="0"/>
         <v>feed_water_tank_zo</v>
       </c>
       <c r="C32" t="s">
+        <v>280</v>
+      </c>
+      <c r="D32" t="s">
         <v>281</v>
       </c>
-      <c r="D32" t="s">
-        <v>282</v>
-      </c>
       <c r="E32" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G32" t="str">
         <f>CONCATENATE(C32," ",D32," ",E32)</f>
@@ -5805,14 +5767,14 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B33" t="str">
         <f t="shared" si="0"/>
         <v>feed_zo</v>
       </c>
       <c r="C33" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="G33" t="str">
         <f t="shared" si="1"/>
@@ -5821,17 +5783,17 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B34" t="str">
         <f t="shared" si="0"/>
         <v>filter_press_zo</v>
       </c>
       <c r="C34" t="s">
+        <v>283</v>
+      </c>
+      <c r="D34" t="s">
         <v>284</v>
-      </c>
-      <c r="D34" t="s">
-        <v>285</v>
       </c>
       <c r="G34" t="str">
         <f t="shared" si="1"/>
@@ -5840,17 +5802,17 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B35" t="str">
         <f t="shared" si="0"/>
         <v>fixed_bed_zo</v>
       </c>
       <c r="C35" t="s">
+        <v>286</v>
+      </c>
+      <c r="D35" t="s">
         <v>287</v>
-      </c>
-      <c r="D35" t="s">
-        <v>288</v>
       </c>
       <c r="G35" t="str">
         <f t="shared" si="1"/>
@@ -5859,14 +5821,14 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B36" t="str">
         <f t="shared" si="0"/>
         <v>gac_zo</v>
       </c>
       <c r="C36" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G36" t="str">
         <f t="shared" si="1"/>
@@ -5875,20 +5837,20 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B37" t="str">
         <f t="shared" si="0"/>
         <v>gas_sparged_membrane_zo</v>
       </c>
       <c r="C37" t="s">
+        <v>290</v>
+      </c>
+      <c r="D37" t="s">
         <v>291</v>
       </c>
-      <c r="D37" t="s">
+      <c r="E37" t="s">
         <v>292</v>
-      </c>
-      <c r="E37" t="s">
-        <v>293</v>
       </c>
       <c r="G37" t="str">
         <f>CONCATENATE(C37," ",D37," ",E37)</f>
@@ -5897,20 +5859,20 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B38" t="str">
         <f t="shared" si="0"/>
         <v>injection_well_disposal_zo</v>
       </c>
       <c r="C38" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D38" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E38" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="G38" t="str">
         <f>CONCATENATE(C38," ",D38," ",E38)</f>
@@ -5919,17 +5881,17 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B39" t="str">
         <f t="shared" si="0"/>
         <v>intrusion_mitigation_zo</v>
       </c>
       <c r="C39" t="s">
+        <v>296</v>
+      </c>
+      <c r="D39" t="s">
         <v>297</v>
-      </c>
-      <c r="D39" t="s">
-        <v>298</v>
       </c>
       <c r="G39" t="str">
         <f t="shared" si="1"/>
@@ -5938,17 +5900,17 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B40" t="str">
         <f t="shared" si="0"/>
         <v>ion_exchange_zo</v>
       </c>
       <c r="C40" t="s">
+        <v>299</v>
+      </c>
+      <c r="D40" t="s">
         <v>300</v>
-      </c>
-      <c r="D40" t="s">
-        <v>301</v>
       </c>
       <c r="G40" t="str">
         <f t="shared" si="1"/>
@@ -5957,23 +5919,23 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B41" t="str">
         <f t="shared" si="0"/>
         <v>iron_and_manganese_removal_zo</v>
       </c>
       <c r="C41" t="s">
+        <v>302</v>
+      </c>
+      <c r="D41" t="s">
+        <v>241</v>
+      </c>
+      <c r="E41" t="s">
         <v>303</v>
       </c>
-      <c r="D41" t="s">
-        <v>242</v>
-      </c>
-      <c r="E41" t="s">
-        <v>304</v>
-      </c>
       <c r="F41" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="G41" t="str">
         <f>CONCATENATE(C41," ",D41," ",E41," ",F41)</f>
@@ -5982,14 +5944,14 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B42" t="str">
         <f t="shared" si="0"/>
         <v>landfill_zo</v>
       </c>
       <c r="C42" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G42" t="str">
         <f t="shared" si="1"/>
@@ -5998,14 +5960,14 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B43" t="str">
         <f t="shared" si="0"/>
         <v>mabr_zo</v>
       </c>
       <c r="C43" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G43" t="str">
         <f t="shared" si="1"/>
@@ -6014,14 +5976,14 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B44" t="str">
         <f t="shared" si="0"/>
         <v>mbr_zo</v>
       </c>
       <c r="C44" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G44" t="str">
         <f t="shared" si="1"/>
@@ -6030,17 +5992,17 @@
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B45" t="str">
         <f t="shared" si="0"/>
         <v>media_filtration_zo</v>
       </c>
       <c r="C45" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D45" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G45" t="str">
         <f t="shared" si="1"/>
@@ -6049,14 +6011,14 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B46" t="str">
         <f t="shared" si="0"/>
         <v>metab_zo</v>
       </c>
       <c r="C46" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G46" t="str">
         <f t="shared" si="1"/>
@@ -6065,14 +6027,14 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B47" t="str">
         <f t="shared" si="0"/>
         <v>microfiltration_zo</v>
       </c>
       <c r="C47" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G47" t="str">
         <f t="shared" si="1"/>
@@ -6081,17 +6043,17 @@
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B48" t="str">
         <f t="shared" si="0"/>
         <v>microscreen_filtration_zo</v>
       </c>
       <c r="C48" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="D48" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G48" t="str">
         <f t="shared" si="1"/>
@@ -6100,17 +6062,17 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B49" t="str">
         <f t="shared" si="0"/>
         <v>municipal_drinking_zo</v>
       </c>
       <c r="C49" t="s">
+        <v>312</v>
+      </c>
+      <c r="D49" t="s">
         <v>313</v>
-      </c>
-      <c r="D49" t="s">
-        <v>314</v>
       </c>
       <c r="G49" t="str">
         <f t="shared" si="1"/>
@@ -6119,17 +6081,17 @@
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B50" t="str">
         <f t="shared" si="0"/>
         <v>municipal_wwtp_zo</v>
       </c>
       <c r="C50" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D50" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="G50" t="str">
         <f t="shared" si="1"/>
@@ -6138,14 +6100,14 @@
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B51" t="str">
         <f t="shared" si="0"/>
         <v>nanofiltration_zo</v>
       </c>
       <c r="C51" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="G51" t="str">
         <f t="shared" si="1"/>
@@ -6154,17 +6116,17 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B52" t="str">
         <f t="shared" si="0"/>
         <v>ozone_aop _zo</v>
       </c>
       <c r="C52" t="s">
+        <v>318</v>
+      </c>
+      <c r="D52" t="s">
         <v>319</v>
-      </c>
-      <c r="D52" t="s">
-        <v>320</v>
       </c>
       <c r="G52" t="str">
         <f t="shared" si="1"/>
@@ -6173,14 +6135,14 @@
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B53" t="str">
         <f t="shared" si="0"/>
         <v>ozone_zo</v>
       </c>
       <c r="C53" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G53" t="str">
         <f t="shared" si="1"/>
@@ -6189,17 +6151,17 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B54" t="str">
         <f t="shared" si="0"/>
         <v>photothermal_membrane_zo</v>
       </c>
       <c r="C54" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D54" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G54" t="str">
         <f t="shared" si="1"/>
@@ -6208,17 +6170,17 @@
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B55" t="str">
         <f t="shared" si="0"/>
         <v>primary_separator_zo</v>
       </c>
       <c r="C55" t="s">
+        <v>323</v>
+      </c>
+      <c r="D55" t="s">
         <v>324</v>
-      </c>
-      <c r="D55" t="s">
-        <v>325</v>
       </c>
       <c r="G55" t="str">
         <f t="shared" si="1"/>
@@ -6234,10 +6196,10 @@
         <v>pump_electricity_zo</v>
       </c>
       <c r="C56" t="s">
+        <v>325</v>
+      </c>
+      <c r="D56" t="s">
         <v>326</v>
-      </c>
-      <c r="D56" t="s">
-        <v>327</v>
       </c>
       <c r="G56" t="str">
         <f t="shared" si="1"/>
@@ -6246,14 +6208,14 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B57" t="str">
         <f t="shared" si="0"/>
         <v>pump_zo</v>
       </c>
       <c r="C57" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G57" t="str">
         <f t="shared" si="1"/>
@@ -6262,14 +6224,14 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B58" t="str">
         <f t="shared" si="0"/>
         <v>screen_zo</v>
       </c>
       <c r="C58" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="G58" t="str">
         <f t="shared" si="1"/>
@@ -6278,20 +6240,20 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B59" t="str">
         <f t="shared" si="0"/>
         <v>secondary_treatment_wwtp_zo</v>
       </c>
       <c r="C59" t="s">
+        <v>329</v>
+      </c>
+      <c r="D59" t="s">
         <v>330</v>
       </c>
-      <c r="D59" t="s">
-        <v>331</v>
-      </c>
       <c r="E59" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="G59" t="str">
         <f>CONCATENATE(C59," ",D59," ",E59)</f>
@@ -6300,14 +6262,14 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B60" t="str">
         <f t="shared" si="0"/>
         <v>sedimentation_zo</v>
       </c>
       <c r="C60" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="G60" t="str">
         <f t="shared" si="1"/>
@@ -6316,17 +6278,17 @@
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B61" t="str">
         <f t="shared" si="0"/>
         <v>settling_pond_zo</v>
       </c>
       <c r="C61" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D61" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="G61" t="str">
         <f t="shared" si="1"/>
@@ -6335,17 +6297,17 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B62" t="str">
         <f t="shared" si="0"/>
         <v>sludge_tank_zo</v>
       </c>
       <c r="C62" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D62" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G62" t="str">
         <f t="shared" si="1"/>
@@ -6354,14 +6316,14 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B63" t="str">
         <f t="shared" si="0"/>
         <v>smp_zo</v>
       </c>
       <c r="C63" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="G63" t="str">
         <f t="shared" si="1"/>
@@ -6370,17 +6332,17 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B64" t="str">
         <f t="shared" si="0"/>
         <v>static_mixer_zo</v>
       </c>
       <c r="C64" t="s">
+        <v>337</v>
+      </c>
+      <c r="D64" t="s">
         <v>338</v>
-      </c>
-      <c r="D64" t="s">
-        <v>339</v>
       </c>
       <c r="G64" t="str">
         <f t="shared" si="1"/>
@@ -6389,17 +6351,17 @@
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B65" t="str">
         <f t="shared" si="0"/>
         <v>storage_tank_zo</v>
       </c>
       <c r="C65" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D65" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G65" t="str">
         <f t="shared" si="1"/>
@@ -6408,17 +6370,17 @@
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B66" t="str">
         <f t="shared" ref="B66:B77" si="6">CONCATENATE(A66,"_zo")</f>
         <v>surface_discharge_zo</v>
       </c>
       <c r="C66" t="s">
+        <v>342</v>
+      </c>
+      <c r="D66" t="s">
         <v>343</v>
-      </c>
-      <c r="D66" t="s">
-        <v>344</v>
       </c>
       <c r="G66" t="str">
         <f t="shared" ref="G66:G77" si="7">CONCATENATE(C66," ",D66)</f>
@@ -6427,20 +6389,20 @@
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B67" t="str">
         <f t="shared" si="6"/>
         <v>sw_onshore_intake_zo</v>
       </c>
       <c r="C67" t="s">
+        <v>345</v>
+      </c>
+      <c r="D67" t="s">
         <v>346</v>
       </c>
-      <c r="D67" t="s">
+      <c r="E67" t="s">
         <v>347</v>
-      </c>
-      <c r="E67" t="s">
-        <v>348</v>
       </c>
       <c r="G67" t="str">
         <f>CONCATENATE(C67," ",D67," ",E67)</f>
@@ -6449,20 +6411,20 @@
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B68" t="str">
         <f t="shared" si="6"/>
         <v>tramp_oil_tank_zo</v>
       </c>
       <c r="C68" t="s">
+        <v>349</v>
+      </c>
+      <c r="D68" t="s">
         <v>350</v>
       </c>
-      <c r="D68" t="s">
-        <v>351</v>
-      </c>
       <c r="E68" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G68" t="str">
         <f t="shared" ref="G68:G69" si="8">CONCATENATE(C68," ",D68," ",E68)</f>
@@ -6471,20 +6433,20 @@
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B69" t="str">
         <f t="shared" si="6"/>
         <v>tri_media_filtration_zo</v>
       </c>
       <c r="C69" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D69" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E69" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G69" t="str">
         <f t="shared" si="8"/>
@@ -6493,17 +6455,17 @@
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B70" t="str">
         <f t="shared" si="6"/>
         <v>ultra_filtration_zo</v>
       </c>
       <c r="C70" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D70" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G70" t="str">
         <f t="shared" si="7"/>
@@ -6512,17 +6474,17 @@
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B71" t="str">
         <f t="shared" si="6"/>
         <v>uv_aop_zo</v>
       </c>
       <c r="C71" t="s">
+        <v>356</v>
+      </c>
+      <c r="D71" t="s">
         <v>357</v>
-      </c>
-      <c r="D71" t="s">
-        <v>358</v>
       </c>
       <c r="G71" t="str">
         <f t="shared" si="7"/>
@@ -6531,14 +6493,14 @@
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B72" t="str">
         <f t="shared" si="6"/>
         <v>uv_zo</v>
       </c>
       <c r="C72" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="G72" t="str">
         <f t="shared" si="7"/>
@@ -6547,17 +6509,17 @@
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B73" t="str">
         <f t="shared" si="6"/>
         <v>vfa_recovery_zo</v>
       </c>
       <c r="C73" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D73" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="G73" t="str">
         <f t="shared" si="7"/>
@@ -6566,14 +6528,14 @@
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B74" t="str">
         <f t="shared" si="6"/>
         <v>waiv_zo</v>
       </c>
       <c r="C74" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="G74" t="str">
         <f t="shared" si="7"/>
@@ -6582,20 +6544,20 @@
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B75" t="str">
         <f t="shared" si="6"/>
         <v>walnut_shell_filter_zo</v>
       </c>
       <c r="C75" t="s">
+        <v>362</v>
+      </c>
+      <c r="D75" t="s">
         <v>363</v>
       </c>
-      <c r="D75" t="s">
-        <v>364</v>
-      </c>
       <c r="E75" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G75" t="str">
         <f t="shared" ref="G75:G76" si="9">CONCATENATE(C75," ",D75," ",E75)</f>
@@ -6604,20 +6566,20 @@
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B76" t="str">
         <f t="shared" si="6"/>
         <v>water_pumping_station_zo</v>
       </c>
       <c r="C76" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D76" t="s">
+        <v>365</v>
+      </c>
+      <c r="E76" t="s">
         <v>366</v>
-      </c>
-      <c r="E76" t="s">
-        <v>367</v>
       </c>
       <c r="G76" t="str">
         <f t="shared" si="9"/>
@@ -6626,17 +6588,17 @@
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="6"/>
         <v>well_field_zo</v>
       </c>
       <c r="C77" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D77" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="G77" t="str">
         <f t="shared" si="7"/>
@@ -6662,7 +6624,7 @@
         <v>9</v>
       </c>
       <c r="C1" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="2" spans="2:3" x14ac:dyDescent="0.2">
@@ -6670,7 +6632,7 @@
         <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.2">
@@ -6678,7 +6640,7 @@
         <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.2">
@@ -6686,15 +6648,15 @@
         <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C5" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.2">
@@ -6702,7 +6664,7 @@
         <v>20</v>
       </c>
       <c r="C6" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.2">
@@ -6710,7 +6672,7 @@
         <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.2">
@@ -6718,15 +6680,15 @@
         <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C9" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.2">
@@ -6734,7 +6696,7 @@
         <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.2">
@@ -6742,7 +6704,7 @@
         <v>34</v>
       </c>
       <c r="C11" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.2">
@@ -6750,7 +6712,7 @@
         <v>36</v>
       </c>
       <c r="C12" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.2">
@@ -6758,7 +6720,7 @@
         <v>39</v>
       </c>
       <c r="C13" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="14" spans="2:3" x14ac:dyDescent="0.2">
@@ -6766,7 +6728,7 @@
         <v>41</v>
       </c>
       <c r="C14" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="15" spans="2:3" x14ac:dyDescent="0.2">
@@ -6774,7 +6736,7 @@
         <v>44</v>
       </c>
       <c r="C15" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.2">
@@ -6782,7 +6744,7 @@
         <v>47</v>
       </c>
       <c r="C16" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.2">
@@ -6790,7 +6752,7 @@
         <v>49</v>
       </c>
       <c r="C17" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
@@ -6798,7 +6760,7 @@
         <v>51</v>
       </c>
       <c r="C18" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.2">
@@ -6806,7 +6768,7 @@
         <v>54</v>
       </c>
       <c r="C19" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
@@ -6814,7 +6776,7 @@
         <v>56</v>
       </c>
       <c r="C20" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
@@ -6822,7 +6784,7 @@
         <v>60</v>
       </c>
       <c r="C21" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
@@ -6830,7 +6792,7 @@
         <v>62</v>
       </c>
       <c r="C22" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.2">
@@ -6838,7 +6800,7 @@
         <v>64</v>
       </c>
       <c r="C23" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.2">
@@ -6846,7 +6808,7 @@
         <v>67</v>
       </c>
       <c r="C24" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
@@ -6854,7 +6816,7 @@
         <v>69</v>
       </c>
       <c r="C25" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="26" spans="2:3" x14ac:dyDescent="0.2">
@@ -6862,7 +6824,7 @@
         <v>72</v>
       </c>
       <c r="C26" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.2">
@@ -6870,7 +6832,7 @@
         <v>74</v>
       </c>
       <c r="C27" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.2">
@@ -6878,7 +6840,7 @@
         <v>77</v>
       </c>
       <c r="C28" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="29" spans="2:3" x14ac:dyDescent="0.2">
@@ -6886,7 +6848,7 @@
         <v>79</v>
       </c>
       <c r="C29" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="30" spans="2:3" x14ac:dyDescent="0.2">
@@ -6894,7 +6856,7 @@
         <v>82</v>
       </c>
       <c r="C30" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="31" spans="2:3" x14ac:dyDescent="0.2">
@@ -6902,7 +6864,7 @@
         <v>84</v>
       </c>
       <c r="C31" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="32" spans="2:3" x14ac:dyDescent="0.2">
@@ -6910,7 +6872,7 @@
         <v>86</v>
       </c>
       <c r="C32" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.2">
@@ -6918,7 +6880,7 @@
         <v>89</v>
       </c>
       <c r="C33" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.2">
@@ -6926,7 +6888,7 @@
         <v>91</v>
       </c>
       <c r="C34" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.2">
@@ -6934,7 +6896,7 @@
         <v>95</v>
       </c>
       <c r="C35" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.2">
@@ -6942,7 +6904,7 @@
         <v>98</v>
       </c>
       <c r="C36" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="37" spans="2:3" x14ac:dyDescent="0.2">
@@ -6950,7 +6912,7 @@
         <v>101</v>
       </c>
       <c r="C37" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.2">
@@ -6958,15 +6920,15 @@
         <v>103</v>
       </c>
       <c r="C38" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="39" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B39" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="C39" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="40" spans="2:3" x14ac:dyDescent="0.2">
@@ -6974,7 +6936,7 @@
         <v>105</v>
       </c>
       <c r="C40" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.2">
@@ -6982,7 +6944,7 @@
         <v>107</v>
       </c>
       <c r="C41" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="42" spans="2:3" x14ac:dyDescent="0.2">
@@ -6990,7 +6952,7 @@
         <v>109</v>
       </c>
       <c r="C42" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="43" spans="2:3" x14ac:dyDescent="0.2">
@@ -6998,7 +6960,7 @@
         <v>112</v>
       </c>
       <c r="C43" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="44" spans="2:3" x14ac:dyDescent="0.2">
@@ -7006,7 +6968,7 @@
         <v>115</v>
       </c>
       <c r="C44" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="45" spans="2:3" x14ac:dyDescent="0.2">
@@ -7014,7 +6976,7 @@
         <v>118</v>
       </c>
       <c r="C45" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="46" spans="2:3" x14ac:dyDescent="0.2">
@@ -7022,7 +6984,7 @@
         <v>121</v>
       </c>
       <c r="C46" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="47" spans="2:3" x14ac:dyDescent="0.2">
@@ -7030,7 +6992,7 @@
         <v>123</v>
       </c>
       <c r="C47" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="48" spans="2:3" x14ac:dyDescent="0.2">
@@ -7038,7 +7000,7 @@
         <v>125</v>
       </c>
       <c r="C48" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.2">
@@ -7046,255 +7008,255 @@
         <v>128</v>
       </c>
       <c r="C49" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="50" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B50" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C50" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="51" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B51" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C51" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B52" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C52" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="53" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B53" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C53" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="54" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B54" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C54" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B55" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C55" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="56" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B56" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C56" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="57" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B57" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C57" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="58" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B58" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C58" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="59" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B59" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C59" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B60" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C60" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="61" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B61" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C61" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="62" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B62" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C62" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B63" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C63" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="64" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B64" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C64" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="65" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B65" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C65" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B66" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C66" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="67" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B67" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C67" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="68" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B68" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C68" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="69" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B69" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C69" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B70" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C70" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="71" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B71" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C71" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="72" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B72" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C72" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="73" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B73" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C73" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="74" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B74" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C74" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="75" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B75" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C75" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="76" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B76" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C76" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="77" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B77" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C77" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="78" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B78" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C78" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="79" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B79" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C79" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="80" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B80" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C80" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
   </sheetData>

</xml_diff>